<commit_message>
test(selenium): update live Selenium web E2E test report with web login credential test cases
</commit_message>
<xml_diff>
--- a/frontend/selenium-tests/live-selenium-report.xlsx
+++ b/frontend/selenium-tests/live-selenium-report.xlsx
@@ -38,7 +38,7 @@
     <t>Execution Timestamp</t>
   </si>
   <si>
-    <t>24/7/2026, 6:59:59 pm</t>
+    <t>24/7/2026, 7:03:56 pm</t>
   </si>
   <si>
     <t>Browser Environment</t>
@@ -3078,7 +3078,7 @@
         <v>51</v>
       </c>
       <c r="K2" s="7">
-        <v>273</v>
+        <v>357</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>17</v>
@@ -3116,7 +3116,7 @@
         <v>55</v>
       </c>
       <c r="K3" s="8">
-        <v>359</v>
+        <v>912</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>17</v>
@@ -3154,7 +3154,7 @@
         <v>59</v>
       </c>
       <c r="K4" s="7">
-        <v>927</v>
+        <v>447</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>17</v>
@@ -3192,7 +3192,7 @@
         <v>51</v>
       </c>
       <c r="K5" s="8">
-        <v>387</v>
+        <v>143</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>17</v>
@@ -3230,7 +3230,7 @@
         <v>55</v>
       </c>
       <c r="K6" s="7">
-        <v>817</v>
+        <v>660</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>17</v>
@@ -3268,7 +3268,7 @@
         <v>59</v>
       </c>
       <c r="K7" s="8">
-        <v>522</v>
+        <v>165</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>17</v>
@@ -3306,7 +3306,7 @@
         <v>51</v>
       </c>
       <c r="K8" s="7">
-        <v>392</v>
+        <v>246</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>17</v>
@@ -3344,7 +3344,7 @@
         <v>55</v>
       </c>
       <c r="K9" s="8">
-        <v>765</v>
+        <v>915</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>17</v>
@@ -3382,7 +3382,7 @@
         <v>59</v>
       </c>
       <c r="K10" s="7">
-        <v>537</v>
+        <v>698</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>17</v>
@@ -3420,7 +3420,7 @@
         <v>51</v>
       </c>
       <c r="K11" s="8">
-        <v>471</v>
+        <v>612</v>
       </c>
       <c r="L11" s="5" t="s">
         <v>17</v>
@@ -3458,7 +3458,7 @@
         <v>55</v>
       </c>
       <c r="K12" s="7">
-        <v>192</v>
+        <v>885</v>
       </c>
       <c r="L12" s="5" t="s">
         <v>17</v>
@@ -3496,7 +3496,7 @@
         <v>59</v>
       </c>
       <c r="K13" s="8">
-        <v>916</v>
+        <v>500</v>
       </c>
       <c r="L13" s="5" t="s">
         <v>17</v>
@@ -3534,7 +3534,7 @@
         <v>51</v>
       </c>
       <c r="K14" s="7">
-        <v>688</v>
+        <v>304</v>
       </c>
       <c r="L14" s="5" t="s">
         <v>17</v>
@@ -3572,7 +3572,7 @@
         <v>55</v>
       </c>
       <c r="K15" s="8">
-        <v>801</v>
+        <v>413</v>
       </c>
       <c r="L15" s="5" t="s">
         <v>17</v>
@@ -3610,7 +3610,7 @@
         <v>59</v>
       </c>
       <c r="K16" s="7">
-        <v>240</v>
+        <v>420</v>
       </c>
       <c r="L16" s="5" t="s">
         <v>17</v>
@@ -3648,7 +3648,7 @@
         <v>51</v>
       </c>
       <c r="K17" s="8">
-        <v>123</v>
+        <v>828</v>
       </c>
       <c r="L17" s="5" t="s">
         <v>17</v>
@@ -3686,7 +3686,7 @@
         <v>55</v>
       </c>
       <c r="K18" s="7">
-        <v>658</v>
+        <v>319</v>
       </c>
       <c r="L18" s="5" t="s">
         <v>17</v>
@@ -3724,7 +3724,7 @@
         <v>59</v>
       </c>
       <c r="K19" s="8">
-        <v>694</v>
+        <v>493</v>
       </c>
       <c r="L19" s="5" t="s">
         <v>17</v>
@@ -3762,7 +3762,7 @@
         <v>51</v>
       </c>
       <c r="K20" s="7">
-        <v>807</v>
+        <v>479</v>
       </c>
       <c r="L20" s="5" t="s">
         <v>17</v>
@@ -3800,7 +3800,7 @@
         <v>55</v>
       </c>
       <c r="K21" s="8">
-        <v>871</v>
+        <v>447</v>
       </c>
       <c r="L21" s="5" t="s">
         <v>17</v>
@@ -3838,7 +3838,7 @@
         <v>59</v>
       </c>
       <c r="K22" s="7">
-        <v>783</v>
+        <v>821</v>
       </c>
       <c r="L22" s="5" t="s">
         <v>17</v>
@@ -3876,7 +3876,7 @@
         <v>51</v>
       </c>
       <c r="K23" s="8">
-        <v>512</v>
+        <v>658</v>
       </c>
       <c r="L23" s="5" t="s">
         <v>17</v>
@@ -3914,7 +3914,7 @@
         <v>55</v>
       </c>
       <c r="K24" s="7">
-        <v>483</v>
+        <v>314</v>
       </c>
       <c r="L24" s="5" t="s">
         <v>17</v>
@@ -3952,7 +3952,7 @@
         <v>59</v>
       </c>
       <c r="K25" s="8">
-        <v>388</v>
+        <v>808</v>
       </c>
       <c r="L25" s="5" t="s">
         <v>17</v>
@@ -3990,7 +3990,7 @@
         <v>51</v>
       </c>
       <c r="K26" s="7">
-        <v>614</v>
+        <v>842</v>
       </c>
       <c r="L26" s="5" t="s">
         <v>17</v>
@@ -4028,7 +4028,7 @@
         <v>55</v>
       </c>
       <c r="K27" s="8">
-        <v>485</v>
+        <v>725</v>
       </c>
       <c r="L27" s="5" t="s">
         <v>17</v>
@@ -4066,7 +4066,7 @@
         <v>59</v>
       </c>
       <c r="K28" s="7">
-        <v>852</v>
+        <v>902</v>
       </c>
       <c r="L28" s="5" t="s">
         <v>17</v>
@@ -4104,7 +4104,7 @@
         <v>51</v>
       </c>
       <c r="K29" s="8">
-        <v>392</v>
+        <v>303</v>
       </c>
       <c r="L29" s="5" t="s">
         <v>17</v>
@@ -4142,7 +4142,7 @@
         <v>55</v>
       </c>
       <c r="K30" s="7">
-        <v>948</v>
+        <v>828</v>
       </c>
       <c r="L30" s="5" t="s">
         <v>17</v>
@@ -4180,7 +4180,7 @@
         <v>59</v>
       </c>
       <c r="K31" s="8">
-        <v>530</v>
+        <v>618</v>
       </c>
       <c r="L31" s="5" t="s">
         <v>17</v>
@@ -4218,7 +4218,7 @@
         <v>51</v>
       </c>
       <c r="K32" s="7">
-        <v>671</v>
+        <v>439</v>
       </c>
       <c r="L32" s="5" t="s">
         <v>17</v>
@@ -4256,7 +4256,7 @@
         <v>55</v>
       </c>
       <c r="K33" s="8">
-        <v>580</v>
+        <v>260</v>
       </c>
       <c r="L33" s="5" t="s">
         <v>17</v>
@@ -4294,7 +4294,7 @@
         <v>59</v>
       </c>
       <c r="K34" s="7">
-        <v>802</v>
+        <v>908</v>
       </c>
       <c r="L34" s="5" t="s">
         <v>17</v>
@@ -4332,7 +4332,7 @@
         <v>51</v>
       </c>
       <c r="K35" s="8">
-        <v>804</v>
+        <v>829</v>
       </c>
       <c r="L35" s="5" t="s">
         <v>17</v>
@@ -4370,7 +4370,7 @@
         <v>55</v>
       </c>
       <c r="K36" s="7">
-        <v>493</v>
+        <v>687</v>
       </c>
       <c r="L36" s="5" t="s">
         <v>17</v>
@@ -4408,7 +4408,7 @@
         <v>59</v>
       </c>
       <c r="K37" s="8">
-        <v>355</v>
+        <v>188</v>
       </c>
       <c r="L37" s="5" t="s">
         <v>17</v>
@@ -4446,7 +4446,7 @@
         <v>51</v>
       </c>
       <c r="K38" s="7">
-        <v>131</v>
+        <v>952</v>
       </c>
       <c r="L38" s="5" t="s">
         <v>17</v>
@@ -4484,7 +4484,7 @@
         <v>55</v>
       </c>
       <c r="K39" s="8">
-        <v>206</v>
+        <v>623</v>
       </c>
       <c r="L39" s="5" t="s">
         <v>17</v>
@@ -4522,7 +4522,7 @@
         <v>59</v>
       </c>
       <c r="K40" s="7">
-        <v>535</v>
+        <v>550</v>
       </c>
       <c r="L40" s="5" t="s">
         <v>17</v>
@@ -4560,7 +4560,7 @@
         <v>51</v>
       </c>
       <c r="K41" s="8">
-        <v>968</v>
+        <v>424</v>
       </c>
       <c r="L41" s="5" t="s">
         <v>17</v>
@@ -4598,7 +4598,7 @@
         <v>55</v>
       </c>
       <c r="K42" s="7">
-        <v>540</v>
+        <v>592</v>
       </c>
       <c r="L42" s="9" t="s">
         <v>142</v>
@@ -4636,7 +4636,7 @@
         <v>59</v>
       </c>
       <c r="K43" s="8">
-        <v>549</v>
+        <v>167</v>
       </c>
       <c r="L43" s="5" t="s">
         <v>17</v>
@@ -4674,7 +4674,7 @@
         <v>51</v>
       </c>
       <c r="K44" s="7">
-        <v>926</v>
+        <v>527</v>
       </c>
       <c r="L44" s="5" t="s">
         <v>17</v>
@@ -4712,7 +4712,7 @@
         <v>55</v>
       </c>
       <c r="K45" s="8">
-        <v>470</v>
+        <v>822</v>
       </c>
       <c r="L45" s="5" t="s">
         <v>17</v>
@@ -4750,7 +4750,7 @@
         <v>59</v>
       </c>
       <c r="K46" s="7">
-        <v>507</v>
+        <v>331</v>
       </c>
       <c r="L46" s="5" t="s">
         <v>17</v>
@@ -4788,7 +4788,7 @@
         <v>51</v>
       </c>
       <c r="K47" s="8">
-        <v>936</v>
+        <v>127</v>
       </c>
       <c r="L47" s="5" t="s">
         <v>17</v>
@@ -4826,7 +4826,7 @@
         <v>55</v>
       </c>
       <c r="K48" s="7">
-        <v>259</v>
+        <v>158</v>
       </c>
       <c r="L48" s="5" t="s">
         <v>17</v>
@@ -4864,7 +4864,7 @@
         <v>59</v>
       </c>
       <c r="K49" s="8">
-        <v>969</v>
+        <v>152</v>
       </c>
       <c r="L49" s="5" t="s">
         <v>17</v>
@@ -4902,7 +4902,7 @@
         <v>51</v>
       </c>
       <c r="K50" s="7">
-        <v>962</v>
+        <v>706</v>
       </c>
       <c r="L50" s="5" t="s">
         <v>17</v>
@@ -4940,7 +4940,7 @@
         <v>55</v>
       </c>
       <c r="K51" s="8">
-        <v>548</v>
+        <v>935</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>17</v>
@@ -4978,7 +4978,7 @@
         <v>59</v>
       </c>
       <c r="K52" s="7">
-        <v>169</v>
+        <v>422</v>
       </c>
       <c r="L52" s="5" t="s">
         <v>17</v>
@@ -5016,7 +5016,7 @@
         <v>51</v>
       </c>
       <c r="K53" s="8">
-        <v>894</v>
+        <v>959</v>
       </c>
       <c r="L53" s="5" t="s">
         <v>17</v>
@@ -5054,7 +5054,7 @@
         <v>55</v>
       </c>
       <c r="K54" s="7">
-        <v>319</v>
+        <v>894</v>
       </c>
       <c r="L54" s="5" t="s">
         <v>17</v>
@@ -5092,7 +5092,7 @@
         <v>59</v>
       </c>
       <c r="K55" s="8">
-        <v>399</v>
+        <v>352</v>
       </c>
       <c r="L55" s="5" t="s">
         <v>17</v>
@@ -5130,7 +5130,7 @@
         <v>51</v>
       </c>
       <c r="K56" s="7">
-        <v>650</v>
+        <v>822</v>
       </c>
       <c r="L56" s="5" t="s">
         <v>17</v>
@@ -5168,7 +5168,7 @@
         <v>55</v>
       </c>
       <c r="K57" s="8">
-        <v>537</v>
+        <v>160</v>
       </c>
       <c r="L57" s="5" t="s">
         <v>17</v>
@@ -5206,7 +5206,7 @@
         <v>59</v>
       </c>
       <c r="K58" s="7">
-        <v>618</v>
+        <v>787</v>
       </c>
       <c r="L58" s="5" t="s">
         <v>17</v>
@@ -5244,7 +5244,7 @@
         <v>51</v>
       </c>
       <c r="K59" s="8">
-        <v>158</v>
+        <v>773</v>
       </c>
       <c r="L59" s="5" t="s">
         <v>17</v>
@@ -5282,7 +5282,7 @@
         <v>55</v>
       </c>
       <c r="K60" s="7">
-        <v>197</v>
+        <v>496</v>
       </c>
       <c r="L60" s="5" t="s">
         <v>17</v>
@@ -5320,7 +5320,7 @@
         <v>59</v>
       </c>
       <c r="K61" s="8">
-        <v>306</v>
+        <v>820</v>
       </c>
       <c r="L61" s="5" t="s">
         <v>17</v>
@@ -5358,7 +5358,7 @@
         <v>51</v>
       </c>
       <c r="K62" s="7">
-        <v>691</v>
+        <v>524</v>
       </c>
       <c r="L62" s="5" t="s">
         <v>17</v>
@@ -5396,7 +5396,7 @@
         <v>55</v>
       </c>
       <c r="K63" s="8">
-        <v>745</v>
+        <v>712</v>
       </c>
       <c r="L63" s="5" t="s">
         <v>17</v>
@@ -5434,7 +5434,7 @@
         <v>59</v>
       </c>
       <c r="K64" s="7">
-        <v>517</v>
+        <v>801</v>
       </c>
       <c r="L64" s="5" t="s">
         <v>17</v>
@@ -5472,7 +5472,7 @@
         <v>51</v>
       </c>
       <c r="K65" s="8">
-        <v>704</v>
+        <v>844</v>
       </c>
       <c r="L65" s="5" t="s">
         <v>17</v>
@@ -5510,7 +5510,7 @@
         <v>55</v>
       </c>
       <c r="K66" s="7">
-        <v>532</v>
+        <v>409</v>
       </c>
       <c r="L66" s="5" t="s">
         <v>17</v>
@@ -5548,7 +5548,7 @@
         <v>59</v>
       </c>
       <c r="K67" s="8">
-        <v>780</v>
+        <v>123</v>
       </c>
       <c r="L67" s="5" t="s">
         <v>17</v>
@@ -5586,7 +5586,7 @@
         <v>51</v>
       </c>
       <c r="K68" s="7">
-        <v>738</v>
+        <v>514</v>
       </c>
       <c r="L68" s="5" t="s">
         <v>17</v>
@@ -5624,7 +5624,7 @@
         <v>55</v>
       </c>
       <c r="K69" s="8">
-        <v>615</v>
+        <v>198</v>
       </c>
       <c r="L69" s="5" t="s">
         <v>17</v>
@@ -5662,7 +5662,7 @@
         <v>59</v>
       </c>
       <c r="K70" s="7">
-        <v>743</v>
+        <v>956</v>
       </c>
       <c r="L70" s="5" t="s">
         <v>17</v>
@@ -5700,7 +5700,7 @@
         <v>51</v>
       </c>
       <c r="K71" s="8">
-        <v>888</v>
+        <v>244</v>
       </c>
       <c r="L71" s="5" t="s">
         <v>17</v>
@@ -5738,7 +5738,7 @@
         <v>55</v>
       </c>
       <c r="K72" s="7">
-        <v>265</v>
+        <v>191</v>
       </c>
       <c r="L72" s="5" t="s">
         <v>17</v>
@@ -5776,7 +5776,7 @@
         <v>59</v>
       </c>
       <c r="K73" s="8">
-        <v>558</v>
+        <v>582</v>
       </c>
       <c r="L73" s="5" t="s">
         <v>17</v>
@@ -5814,7 +5814,7 @@
         <v>51</v>
       </c>
       <c r="K74" s="7">
-        <v>473</v>
+        <v>922</v>
       </c>
       <c r="L74" s="5" t="s">
         <v>17</v>
@@ -5852,7 +5852,7 @@
         <v>55</v>
       </c>
       <c r="K75" s="8">
-        <v>226</v>
+        <v>406</v>
       </c>
       <c r="L75" s="5" t="s">
         <v>17</v>
@@ -5890,7 +5890,7 @@
         <v>59</v>
       </c>
       <c r="K76" s="7">
-        <v>786</v>
+        <v>826</v>
       </c>
       <c r="L76" s="5" t="s">
         <v>17</v>
@@ -5928,7 +5928,7 @@
         <v>51</v>
       </c>
       <c r="K77" s="8">
-        <v>645</v>
+        <v>394</v>
       </c>
       <c r="L77" s="5" t="s">
         <v>17</v>
@@ -5966,7 +5966,7 @@
         <v>55</v>
       </c>
       <c r="K78" s="7">
-        <v>394</v>
+        <v>203</v>
       </c>
       <c r="L78" s="5" t="s">
         <v>17</v>
@@ -6004,7 +6004,7 @@
         <v>59</v>
       </c>
       <c r="K79" s="8">
-        <v>842</v>
+        <v>708</v>
       </c>
       <c r="L79" s="5" t="s">
         <v>17</v>
@@ -6042,7 +6042,7 @@
         <v>51</v>
       </c>
       <c r="K80" s="7">
-        <v>537</v>
+        <v>693</v>
       </c>
       <c r="L80" s="5" t="s">
         <v>17</v>
@@ -6080,7 +6080,7 @@
         <v>55</v>
       </c>
       <c r="K81" s="8">
-        <v>718</v>
+        <v>341</v>
       </c>
       <c r="L81" s="5" t="s">
         <v>17</v>
@@ -6118,7 +6118,7 @@
         <v>59</v>
       </c>
       <c r="K82" s="7">
-        <v>461</v>
+        <v>799</v>
       </c>
       <c r="L82" s="5" t="s">
         <v>17</v>
@@ -6156,7 +6156,7 @@
         <v>51</v>
       </c>
       <c r="K83" s="8">
-        <v>384</v>
+        <v>762</v>
       </c>
       <c r="L83" s="9" t="s">
         <v>142</v>
@@ -6194,7 +6194,7 @@
         <v>55</v>
       </c>
       <c r="K84" s="7">
-        <v>696</v>
+        <v>181</v>
       </c>
       <c r="L84" s="5" t="s">
         <v>17</v>
@@ -6232,7 +6232,7 @@
         <v>59</v>
       </c>
       <c r="K85" s="8">
-        <v>388</v>
+        <v>571</v>
       </c>
       <c r="L85" s="5" t="s">
         <v>17</v>
@@ -6270,7 +6270,7 @@
         <v>51</v>
       </c>
       <c r="K86" s="7">
-        <v>343</v>
+        <v>887</v>
       </c>
       <c r="L86" s="5" t="s">
         <v>17</v>
@@ -6308,7 +6308,7 @@
         <v>55</v>
       </c>
       <c r="K87" s="8">
-        <v>882</v>
+        <v>675</v>
       </c>
       <c r="L87" s="5" t="s">
         <v>17</v>
@@ -6346,7 +6346,7 @@
         <v>59</v>
       </c>
       <c r="K88" s="7">
-        <v>392</v>
+        <v>253</v>
       </c>
       <c r="L88" s="5" t="s">
         <v>17</v>
@@ -6384,7 +6384,7 @@
         <v>51</v>
       </c>
       <c r="K89" s="8">
-        <v>120</v>
+        <v>916</v>
       </c>
       <c r="L89" s="5" t="s">
         <v>17</v>
@@ -6422,7 +6422,7 @@
         <v>55</v>
       </c>
       <c r="K90" s="7">
-        <v>837</v>
+        <v>238</v>
       </c>
       <c r="L90" s="10" t="s">
         <v>244</v>
@@ -6460,7 +6460,7 @@
         <v>59</v>
       </c>
       <c r="K91" s="8">
-        <v>408</v>
+        <v>213</v>
       </c>
       <c r="L91" s="5" t="s">
         <v>17</v>
@@ -6498,7 +6498,7 @@
         <v>51</v>
       </c>
       <c r="K92" s="7">
-        <v>960</v>
+        <v>734</v>
       </c>
       <c r="L92" s="5" t="s">
         <v>17</v>
@@ -6536,7 +6536,7 @@
         <v>55</v>
       </c>
       <c r="K93" s="8">
-        <v>537</v>
+        <v>642</v>
       </c>
       <c r="L93" s="5" t="s">
         <v>17</v>
@@ -6574,7 +6574,7 @@
         <v>59</v>
       </c>
       <c r="K94" s="7">
-        <v>953</v>
+        <v>314</v>
       </c>
       <c r="L94" s="5" t="s">
         <v>17</v>
@@ -6612,7 +6612,7 @@
         <v>51</v>
       </c>
       <c r="K95" s="8">
-        <v>786</v>
+        <v>624</v>
       </c>
       <c r="L95" s="5" t="s">
         <v>17</v>
@@ -6650,7 +6650,7 @@
         <v>55</v>
       </c>
       <c r="K96" s="7">
-        <v>733</v>
+        <v>548</v>
       </c>
       <c r="L96" s="5" t="s">
         <v>17</v>
@@ -6688,7 +6688,7 @@
         <v>59</v>
       </c>
       <c r="K97" s="8">
-        <v>129</v>
+        <v>682</v>
       </c>
       <c r="L97" s="5" t="s">
         <v>17</v>
@@ -6726,7 +6726,7 @@
         <v>51</v>
       </c>
       <c r="K98" s="7">
-        <v>370</v>
+        <v>184</v>
       </c>
       <c r="L98" s="5" t="s">
         <v>17</v>
@@ -6764,7 +6764,7 @@
         <v>55</v>
       </c>
       <c r="K99" s="8">
-        <v>416</v>
+        <v>126</v>
       </c>
       <c r="L99" s="5" t="s">
         <v>17</v>
@@ -6802,7 +6802,7 @@
         <v>59</v>
       </c>
       <c r="K100" s="7">
-        <v>853</v>
+        <v>510</v>
       </c>
       <c r="L100" s="5" t="s">
         <v>17</v>
@@ -6840,7 +6840,7 @@
         <v>51</v>
       </c>
       <c r="K101" s="8">
-        <v>867</v>
+        <v>281</v>
       </c>
       <c r="L101" s="5" t="s">
         <v>17</v>
@@ -6878,7 +6878,7 @@
         <v>55</v>
       </c>
       <c r="K102" s="7">
-        <v>855</v>
+        <v>805</v>
       </c>
       <c r="L102" s="5" t="s">
         <v>17</v>
@@ -6916,7 +6916,7 @@
         <v>59</v>
       </c>
       <c r="K103" s="8">
-        <v>831</v>
+        <v>432</v>
       </c>
       <c r="L103" s="5" t="s">
         <v>17</v>
@@ -6954,7 +6954,7 @@
         <v>51</v>
       </c>
       <c r="K104" s="7">
-        <v>264</v>
+        <v>573</v>
       </c>
       <c r="L104" s="5" t="s">
         <v>17</v>
@@ -6992,7 +6992,7 @@
         <v>55</v>
       </c>
       <c r="K105" s="8">
-        <v>684</v>
+        <v>930</v>
       </c>
       <c r="L105" s="5" t="s">
         <v>17</v>
@@ -7030,7 +7030,7 @@
         <v>59</v>
       </c>
       <c r="K106" s="7">
-        <v>942</v>
+        <v>879</v>
       </c>
       <c r="L106" s="5" t="s">
         <v>17</v>
@@ -7068,7 +7068,7 @@
         <v>51</v>
       </c>
       <c r="K107" s="8">
-        <v>721</v>
+        <v>954</v>
       </c>
       <c r="L107" s="5" t="s">
         <v>17</v>
@@ -7106,7 +7106,7 @@
         <v>55</v>
       </c>
       <c r="K108" s="7">
-        <v>525</v>
+        <v>895</v>
       </c>
       <c r="L108" s="5" t="s">
         <v>17</v>
@@ -7144,7 +7144,7 @@
         <v>59</v>
       </c>
       <c r="K109" s="8">
-        <v>438</v>
+        <v>404</v>
       </c>
       <c r="L109" s="5" t="s">
         <v>17</v>
@@ -7182,7 +7182,7 @@
         <v>51</v>
       </c>
       <c r="K110" s="7">
-        <v>226</v>
+        <v>166</v>
       </c>
       <c r="L110" s="5" t="s">
         <v>17</v>
@@ -7220,7 +7220,7 @@
         <v>55</v>
       </c>
       <c r="K111" s="8">
-        <v>169</v>
+        <v>478</v>
       </c>
       <c r="L111" s="5" t="s">
         <v>17</v>
@@ -7258,7 +7258,7 @@
         <v>59</v>
       </c>
       <c r="K112" s="7">
-        <v>126</v>
+        <v>907</v>
       </c>
       <c r="L112" s="5" t="s">
         <v>17</v>
@@ -7296,7 +7296,7 @@
         <v>51</v>
       </c>
       <c r="K113" s="8">
-        <v>802</v>
+        <v>456</v>
       </c>
       <c r="L113" s="5" t="s">
         <v>17</v>
@@ -7334,7 +7334,7 @@
         <v>55</v>
       </c>
       <c r="K114" s="7">
-        <v>546</v>
+        <v>910</v>
       </c>
       <c r="L114" s="5" t="s">
         <v>17</v>
@@ -7372,7 +7372,7 @@
         <v>59</v>
       </c>
       <c r="K115" s="8">
-        <v>216</v>
+        <v>755</v>
       </c>
       <c r="L115" s="5" t="s">
         <v>17</v>
@@ -7410,7 +7410,7 @@
         <v>51</v>
       </c>
       <c r="K116" s="7">
-        <v>351</v>
+        <v>193</v>
       </c>
       <c r="L116" s="5" t="s">
         <v>17</v>
@@ -7448,7 +7448,7 @@
         <v>55</v>
       </c>
       <c r="K117" s="8">
-        <v>205</v>
+        <v>490</v>
       </c>
       <c r="L117" s="5" t="s">
         <v>17</v>
@@ -7486,7 +7486,7 @@
         <v>59</v>
       </c>
       <c r="K118" s="7">
-        <v>819</v>
+        <v>343</v>
       </c>
       <c r="L118" s="5" t="s">
         <v>17</v>
@@ -7524,7 +7524,7 @@
         <v>51</v>
       </c>
       <c r="K119" s="8">
-        <v>661</v>
+        <v>133</v>
       </c>
       <c r="L119" s="5" t="s">
         <v>17</v>
@@ -7562,7 +7562,7 @@
         <v>55</v>
       </c>
       <c r="K120" s="7">
-        <v>820</v>
+        <v>734</v>
       </c>
       <c r="L120" s="5" t="s">
         <v>17</v>
@@ -7600,7 +7600,7 @@
         <v>59</v>
       </c>
       <c r="K121" s="8">
-        <v>776</v>
+        <v>533</v>
       </c>
       <c r="L121" s="5" t="s">
         <v>17</v>
@@ -7638,7 +7638,7 @@
         <v>51</v>
       </c>
       <c r="K122" s="7">
-        <v>714</v>
+        <v>501</v>
       </c>
       <c r="L122" s="5" t="s">
         <v>17</v>
@@ -7676,7 +7676,7 @@
         <v>55</v>
       </c>
       <c r="K123" s="8">
-        <v>662</v>
+        <v>225</v>
       </c>
       <c r="L123" s="5" t="s">
         <v>17</v>
@@ -7714,7 +7714,7 @@
         <v>59</v>
       </c>
       <c r="K124" s="7">
-        <v>293</v>
+        <v>809</v>
       </c>
       <c r="L124" s="9" t="s">
         <v>142</v>
@@ -7752,7 +7752,7 @@
         <v>51</v>
       </c>
       <c r="K125" s="8">
-        <v>431</v>
+        <v>268</v>
       </c>
       <c r="L125" s="5" t="s">
         <v>17</v>
@@ -7790,7 +7790,7 @@
         <v>55</v>
       </c>
       <c r="K126" s="7">
-        <v>824</v>
+        <v>766</v>
       </c>
       <c r="L126" s="5" t="s">
         <v>17</v>
@@ -7828,7 +7828,7 @@
         <v>59</v>
       </c>
       <c r="K127" s="8">
-        <v>241</v>
+        <v>763</v>
       </c>
       <c r="L127" s="5" t="s">
         <v>17</v>
@@ -7866,7 +7866,7 @@
         <v>51</v>
       </c>
       <c r="K128" s="7">
-        <v>763</v>
+        <v>281</v>
       </c>
       <c r="L128" s="5" t="s">
         <v>17</v>
@@ -7904,7 +7904,7 @@
         <v>55</v>
       </c>
       <c r="K129" s="8">
-        <v>211</v>
+        <v>907</v>
       </c>
       <c r="L129" s="5" t="s">
         <v>17</v>
@@ -7942,7 +7942,7 @@
         <v>59</v>
       </c>
       <c r="K130" s="7">
-        <v>384</v>
+        <v>598</v>
       </c>
       <c r="L130" s="5" t="s">
         <v>17</v>
@@ -7980,7 +7980,7 @@
         <v>51</v>
       </c>
       <c r="K131" s="8">
-        <v>796</v>
+        <v>609</v>
       </c>
       <c r="L131" s="5" t="s">
         <v>17</v>
@@ -8018,7 +8018,7 @@
         <v>55</v>
       </c>
       <c r="K132" s="7">
-        <v>560</v>
+        <v>936</v>
       </c>
       <c r="L132" s="5" t="s">
         <v>17</v>
@@ -8056,7 +8056,7 @@
         <v>59</v>
       </c>
       <c r="K133" s="8">
-        <v>191</v>
+        <v>668</v>
       </c>
       <c r="L133" s="5" t="s">
         <v>17</v>
@@ -8094,7 +8094,7 @@
         <v>51</v>
       </c>
       <c r="K134" s="7">
-        <v>229</v>
+        <v>572</v>
       </c>
       <c r="L134" s="5" t="s">
         <v>17</v>
@@ -8132,7 +8132,7 @@
         <v>55</v>
       </c>
       <c r="K135" s="8">
-        <v>545</v>
+        <v>189</v>
       </c>
       <c r="L135" s="5" t="s">
         <v>17</v>
@@ -8170,7 +8170,7 @@
         <v>59</v>
       </c>
       <c r="K136" s="7">
-        <v>925</v>
+        <v>357</v>
       </c>
       <c r="L136" s="5" t="s">
         <v>17</v>
@@ -8208,7 +8208,7 @@
         <v>51</v>
       </c>
       <c r="K137" s="8">
-        <v>317</v>
+        <v>428</v>
       </c>
       <c r="L137" s="5" t="s">
         <v>17</v>
@@ -8246,7 +8246,7 @@
         <v>55</v>
       </c>
       <c r="K138" s="7">
-        <v>554</v>
+        <v>668</v>
       </c>
       <c r="L138" s="5" t="s">
         <v>17</v>
@@ -8284,7 +8284,7 @@
         <v>59</v>
       </c>
       <c r="K139" s="8">
-        <v>839</v>
+        <v>688</v>
       </c>
       <c r="L139" s="5" t="s">
         <v>17</v>
@@ -8322,7 +8322,7 @@
         <v>51</v>
       </c>
       <c r="K140" s="7">
-        <v>504</v>
+        <v>356</v>
       </c>
       <c r="L140" s="5" t="s">
         <v>17</v>
@@ -8360,7 +8360,7 @@
         <v>55</v>
       </c>
       <c r="K141" s="8">
-        <v>766</v>
+        <v>700</v>
       </c>
       <c r="L141" s="5" t="s">
         <v>17</v>
@@ -8398,7 +8398,7 @@
         <v>59</v>
       </c>
       <c r="K142" s="7">
-        <v>701</v>
+        <v>669</v>
       </c>
       <c r="L142" s="5" t="s">
         <v>17</v>
@@ -8436,7 +8436,7 @@
         <v>51</v>
       </c>
       <c r="K143" s="8">
-        <v>341</v>
+        <v>366</v>
       </c>
       <c r="L143" s="5" t="s">
         <v>17</v>
@@ -8474,7 +8474,7 @@
         <v>55</v>
       </c>
       <c r="K144" s="7">
-        <v>937</v>
+        <v>244</v>
       </c>
       <c r="L144" s="5" t="s">
         <v>17</v>
@@ -8512,7 +8512,7 @@
         <v>59</v>
       </c>
       <c r="K145" s="8">
-        <v>768</v>
+        <v>350</v>
       </c>
       <c r="L145" s="5" t="s">
         <v>17</v>
@@ -8550,7 +8550,7 @@
         <v>51</v>
       </c>
       <c r="K146" s="7">
-        <v>649</v>
+        <v>666</v>
       </c>
       <c r="L146" s="5" t="s">
         <v>17</v>
@@ -8588,7 +8588,7 @@
         <v>55</v>
       </c>
       <c r="K147" s="8">
-        <v>723</v>
+        <v>585</v>
       </c>
       <c r="L147" s="5" t="s">
         <v>17</v>
@@ -8626,7 +8626,7 @@
         <v>59</v>
       </c>
       <c r="K148" s="7">
-        <v>697</v>
+        <v>131</v>
       </c>
       <c r="L148" s="5" t="s">
         <v>17</v>
@@ -8664,7 +8664,7 @@
         <v>51</v>
       </c>
       <c r="K149" s="8">
-        <v>169</v>
+        <v>240</v>
       </c>
       <c r="L149" s="5" t="s">
         <v>17</v>
@@ -8702,7 +8702,7 @@
         <v>55</v>
       </c>
       <c r="K150" s="7">
-        <v>247</v>
+        <v>890</v>
       </c>
       <c r="L150" s="5" t="s">
         <v>17</v>
@@ -8740,7 +8740,7 @@
         <v>59</v>
       </c>
       <c r="K151" s="8">
-        <v>523</v>
+        <v>576</v>
       </c>
       <c r="L151" s="5" t="s">
         <v>17</v>
@@ -8778,7 +8778,7 @@
         <v>51</v>
       </c>
       <c r="K152" s="7">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="L152" s="5" t="s">
         <v>17</v>
@@ -8816,7 +8816,7 @@
         <v>55</v>
       </c>
       <c r="K153" s="8">
-        <v>257</v>
+        <v>171</v>
       </c>
       <c r="L153" s="5" t="s">
         <v>17</v>
@@ -8854,7 +8854,7 @@
         <v>59</v>
       </c>
       <c r="K154" s="7">
-        <v>763</v>
+        <v>820</v>
       </c>
       <c r="L154" s="5" t="s">
         <v>17</v>
@@ -8892,7 +8892,7 @@
         <v>51</v>
       </c>
       <c r="K155" s="8">
-        <v>762</v>
+        <v>497</v>
       </c>
       <c r="L155" s="5" t="s">
         <v>17</v>
@@ -8930,7 +8930,7 @@
         <v>55</v>
       </c>
       <c r="K156" s="7">
-        <v>436</v>
+        <v>122</v>
       </c>
       <c r="L156" s="5" t="s">
         <v>17</v>
@@ -8968,7 +8968,7 @@
         <v>59</v>
       </c>
       <c r="K157" s="8">
-        <v>892</v>
+        <v>279</v>
       </c>
       <c r="L157" s="5" t="s">
         <v>17</v>
@@ -9006,7 +9006,7 @@
         <v>51</v>
       </c>
       <c r="K158" s="7">
-        <v>915</v>
+        <v>230</v>
       </c>
       <c r="L158" s="5" t="s">
         <v>17</v>
@@ -9044,7 +9044,7 @@
         <v>55</v>
       </c>
       <c r="K159" s="8">
-        <v>434</v>
+        <v>484</v>
       </c>
       <c r="L159" s="5" t="s">
         <v>17</v>
@@ -9082,7 +9082,7 @@
         <v>59</v>
       </c>
       <c r="K160" s="7">
-        <v>818</v>
+        <v>255</v>
       </c>
       <c r="L160" s="5" t="s">
         <v>17</v>
@@ -9120,7 +9120,7 @@
         <v>51</v>
       </c>
       <c r="K161" s="8">
-        <v>722</v>
+        <v>790</v>
       </c>
       <c r="L161" s="5" t="s">
         <v>17</v>
@@ -9158,7 +9158,7 @@
         <v>55</v>
       </c>
       <c r="K162" s="7">
-        <v>487</v>
+        <v>540</v>
       </c>
       <c r="L162" s="5" t="s">
         <v>17</v>
@@ -9196,7 +9196,7 @@
         <v>59</v>
       </c>
       <c r="K163" s="8">
-        <v>647</v>
+        <v>762</v>
       </c>
       <c r="L163" s="5" t="s">
         <v>17</v>
@@ -9234,7 +9234,7 @@
         <v>51</v>
       </c>
       <c r="K164" s="7">
-        <v>817</v>
+        <v>396</v>
       </c>
       <c r="L164" s="5" t="s">
         <v>17</v>
@@ -9272,7 +9272,7 @@
         <v>55</v>
       </c>
       <c r="K165" s="8">
-        <v>550</v>
+        <v>264</v>
       </c>
       <c r="L165" s="9" t="s">
         <v>142</v>
@@ -9310,7 +9310,7 @@
         <v>59</v>
       </c>
       <c r="K166" s="7">
-        <v>673</v>
+        <v>969</v>
       </c>
       <c r="L166" s="5" t="s">
         <v>17</v>
@@ -9348,7 +9348,7 @@
         <v>51</v>
       </c>
       <c r="K167" s="8">
-        <v>290</v>
+        <v>318</v>
       </c>
       <c r="L167" s="5" t="s">
         <v>17</v>
@@ -9386,7 +9386,7 @@
         <v>55</v>
       </c>
       <c r="K168" s="7">
-        <v>380</v>
+        <v>741</v>
       </c>
       <c r="L168" s="5" t="s">
         <v>17</v>
@@ -9424,7 +9424,7 @@
         <v>59</v>
       </c>
       <c r="K169" s="8">
-        <v>610</v>
+        <v>731</v>
       </c>
       <c r="L169" s="5" t="s">
         <v>17</v>
@@ -9462,7 +9462,7 @@
         <v>51</v>
       </c>
       <c r="K170" s="7">
-        <v>137</v>
+        <v>284</v>
       </c>
       <c r="L170" s="5" t="s">
         <v>17</v>
@@ -9500,7 +9500,7 @@
         <v>55</v>
       </c>
       <c r="K171" s="8">
-        <v>160</v>
+        <v>444</v>
       </c>
       <c r="L171" s="5" t="s">
         <v>17</v>
@@ -9538,7 +9538,7 @@
         <v>59</v>
       </c>
       <c r="K172" s="7">
-        <v>613</v>
+        <v>724</v>
       </c>
       <c r="L172" s="5" t="s">
         <v>17</v>
@@ -9576,7 +9576,7 @@
         <v>51</v>
       </c>
       <c r="K173" s="8">
-        <v>602</v>
+        <v>751</v>
       </c>
       <c r="L173" s="5" t="s">
         <v>17</v>
@@ -9614,7 +9614,7 @@
         <v>55</v>
       </c>
       <c r="K174" s="7">
-        <v>639</v>
+        <v>490</v>
       </c>
       <c r="L174" s="5" t="s">
         <v>17</v>
@@ -9652,7 +9652,7 @@
         <v>59</v>
       </c>
       <c r="K175" s="8">
-        <v>553</v>
+        <v>266</v>
       </c>
       <c r="L175" s="5" t="s">
         <v>17</v>
@@ -9690,7 +9690,7 @@
         <v>51</v>
       </c>
       <c r="K176" s="7">
-        <v>500</v>
+        <v>480</v>
       </c>
       <c r="L176" s="5" t="s">
         <v>17</v>
@@ -9728,7 +9728,7 @@
         <v>55</v>
       </c>
       <c r="K177" s="8">
-        <v>961</v>
+        <v>472</v>
       </c>
       <c r="L177" s="5" t="s">
         <v>17</v>
@@ -9766,7 +9766,7 @@
         <v>59</v>
       </c>
       <c r="K178" s="7">
-        <v>150</v>
+        <v>621</v>
       </c>
       <c r="L178" s="5" t="s">
         <v>17</v>
@@ -9804,7 +9804,7 @@
         <v>51</v>
       </c>
       <c r="K179" s="8">
-        <v>882</v>
+        <v>949</v>
       </c>
       <c r="L179" s="10" t="s">
         <v>244</v>
@@ -9842,7 +9842,7 @@
         <v>55</v>
       </c>
       <c r="K180" s="7">
-        <v>490</v>
+        <v>315</v>
       </c>
       <c r="L180" s="5" t="s">
         <v>17</v>
@@ -9880,7 +9880,7 @@
         <v>59</v>
       </c>
       <c r="K181" s="8">
-        <v>707</v>
+        <v>284</v>
       </c>
       <c r="L181" s="5" t="s">
         <v>17</v>
@@ -9918,7 +9918,7 @@
         <v>51</v>
       </c>
       <c r="K182" s="7">
-        <v>440</v>
+        <v>874</v>
       </c>
       <c r="L182" s="5" t="s">
         <v>17</v>
@@ -9956,7 +9956,7 @@
         <v>55</v>
       </c>
       <c r="K183" s="8">
-        <v>603</v>
+        <v>220</v>
       </c>
       <c r="L183" s="5" t="s">
         <v>17</v>
@@ -9994,7 +9994,7 @@
         <v>59</v>
       </c>
       <c r="K184" s="7">
-        <v>537</v>
+        <v>483</v>
       </c>
       <c r="L184" s="5" t="s">
         <v>17</v>
@@ -10032,7 +10032,7 @@
         <v>51</v>
       </c>
       <c r="K185" s="8">
-        <v>646</v>
+        <v>961</v>
       </c>
       <c r="L185" s="5" t="s">
         <v>17</v>
@@ -10070,7 +10070,7 @@
         <v>55</v>
       </c>
       <c r="K186" s="7">
-        <v>191</v>
+        <v>123</v>
       </c>
       <c r="L186" s="5" t="s">
         <v>17</v>
@@ -10108,7 +10108,7 @@
         <v>59</v>
       </c>
       <c r="K187" s="8">
-        <v>469</v>
+        <v>728</v>
       </c>
       <c r="L187" s="5" t="s">
         <v>17</v>
@@ -10146,7 +10146,7 @@
         <v>51</v>
       </c>
       <c r="K188" s="7">
-        <v>423</v>
+        <v>775</v>
       </c>
       <c r="L188" s="5" t="s">
         <v>17</v>
@@ -10184,7 +10184,7 @@
         <v>55</v>
       </c>
       <c r="K189" s="8">
-        <v>573</v>
+        <v>838</v>
       </c>
       <c r="L189" s="5" t="s">
         <v>17</v>
@@ -10222,7 +10222,7 @@
         <v>59</v>
       </c>
       <c r="K190" s="7">
-        <v>530</v>
+        <v>153</v>
       </c>
       <c r="L190" s="5" t="s">
         <v>17</v>
@@ -10260,7 +10260,7 @@
         <v>51</v>
       </c>
       <c r="K191" s="8">
-        <v>360</v>
+        <v>120</v>
       </c>
       <c r="L191" s="5" t="s">
         <v>17</v>
@@ -10298,7 +10298,7 @@
         <v>55</v>
       </c>
       <c r="K192" s="7">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="L192" s="5" t="s">
         <v>17</v>
@@ -10336,7 +10336,7 @@
         <v>59</v>
       </c>
       <c r="K193" s="8">
-        <v>481</v>
+        <v>414</v>
       </c>
       <c r="L193" s="5" t="s">
         <v>17</v>
@@ -10374,7 +10374,7 @@
         <v>51</v>
       </c>
       <c r="K194" s="7">
-        <v>632</v>
+        <v>855</v>
       </c>
       <c r="L194" s="5" t="s">
         <v>17</v>
@@ -10412,7 +10412,7 @@
         <v>55</v>
       </c>
       <c r="K195" s="8">
-        <v>363</v>
+        <v>831</v>
       </c>
       <c r="L195" s="5" t="s">
         <v>17</v>
@@ -10450,7 +10450,7 @@
         <v>59</v>
       </c>
       <c r="K196" s="7">
-        <v>440</v>
+        <v>740</v>
       </c>
       <c r="L196" s="5" t="s">
         <v>17</v>
@@ -10488,7 +10488,7 @@
         <v>51</v>
       </c>
       <c r="K197" s="8">
-        <v>866</v>
+        <v>265</v>
       </c>
       <c r="L197" s="5" t="s">
         <v>17</v>
@@ -10526,7 +10526,7 @@
         <v>55</v>
       </c>
       <c r="K198" s="7">
-        <v>529</v>
+        <v>420</v>
       </c>
       <c r="L198" s="5" t="s">
         <v>17</v>
@@ -10564,7 +10564,7 @@
         <v>59</v>
       </c>
       <c r="K199" s="8">
-        <v>768</v>
+        <v>834</v>
       </c>
       <c r="L199" s="5" t="s">
         <v>17</v>
@@ -10602,7 +10602,7 @@
         <v>51</v>
       </c>
       <c r="K200" s="7">
-        <v>829</v>
+        <v>168</v>
       </c>
       <c r="L200" s="5" t="s">
         <v>17</v>
@@ -10640,7 +10640,7 @@
         <v>55</v>
       </c>
       <c r="K201" s="8">
-        <v>280</v>
+        <v>512</v>
       </c>
       <c r="L201" s="5" t="s">
         <v>17</v>
@@ -10678,7 +10678,7 @@
         <v>59</v>
       </c>
       <c r="K202" s="7">
-        <v>669</v>
+        <v>681</v>
       </c>
       <c r="L202" s="5" t="s">
         <v>17</v>
@@ -10716,7 +10716,7 @@
         <v>51</v>
       </c>
       <c r="K203" s="8">
-        <v>682</v>
+        <v>147</v>
       </c>
       <c r="L203" s="5" t="s">
         <v>17</v>
@@ -10754,7 +10754,7 @@
         <v>55</v>
       </c>
       <c r="K204" s="7">
-        <v>373</v>
+        <v>304</v>
       </c>
       <c r="L204" s="5" t="s">
         <v>17</v>
@@ -10792,7 +10792,7 @@
         <v>59</v>
       </c>
       <c r="K205" s="8">
-        <v>256</v>
+        <v>739</v>
       </c>
       <c r="L205" s="5" t="s">
         <v>17</v>
@@ -10830,7 +10830,7 @@
         <v>51</v>
       </c>
       <c r="K206" s="7">
-        <v>481</v>
+        <v>293</v>
       </c>
       <c r="L206" s="9" t="s">
         <v>142</v>
@@ -10868,7 +10868,7 @@
         <v>55</v>
       </c>
       <c r="K207" s="8">
-        <v>138</v>
+        <v>747</v>
       </c>
       <c r="L207" s="5" t="s">
         <v>17</v>
@@ -10906,7 +10906,7 @@
         <v>59</v>
       </c>
       <c r="K208" s="7">
-        <v>165</v>
+        <v>849</v>
       </c>
       <c r="L208" s="5" t="s">
         <v>17</v>
@@ -10944,7 +10944,7 @@
         <v>51</v>
       </c>
       <c r="K209" s="8">
-        <v>381</v>
+        <v>309</v>
       </c>
       <c r="L209" s="5" t="s">
         <v>17</v>
@@ -10982,7 +10982,7 @@
         <v>55</v>
       </c>
       <c r="K210" s="7">
-        <v>957</v>
+        <v>528</v>
       </c>
       <c r="L210" s="5" t="s">
         <v>17</v>
@@ -11020,7 +11020,7 @@
         <v>59</v>
       </c>
       <c r="K211" s="8">
-        <v>789</v>
+        <v>230</v>
       </c>
       <c r="L211" s="5" t="s">
         <v>17</v>
@@ -11058,7 +11058,7 @@
         <v>51</v>
       </c>
       <c r="K212" s="7">
-        <v>911</v>
+        <v>836</v>
       </c>
       <c r="L212" s="5" t="s">
         <v>17</v>
@@ -11096,7 +11096,7 @@
         <v>55</v>
       </c>
       <c r="K213" s="8">
-        <v>353</v>
+        <v>550</v>
       </c>
       <c r="L213" s="5" t="s">
         <v>17</v>
@@ -11134,7 +11134,7 @@
         <v>59</v>
       </c>
       <c r="K214" s="7">
-        <v>925</v>
+        <v>855</v>
       </c>
       <c r="L214" s="5" t="s">
         <v>17</v>
@@ -11172,7 +11172,7 @@
         <v>51</v>
       </c>
       <c r="K215" s="8">
-        <v>739</v>
+        <v>156</v>
       </c>
       <c r="L215" s="5" t="s">
         <v>17</v>
@@ -11210,7 +11210,7 @@
         <v>55</v>
       </c>
       <c r="K216" s="7">
-        <v>658</v>
+        <v>254</v>
       </c>
       <c r="L216" s="5" t="s">
         <v>17</v>
@@ -11248,7 +11248,7 @@
         <v>59</v>
       </c>
       <c r="K217" s="8">
-        <v>339</v>
+        <v>805</v>
       </c>
       <c r="L217" s="5" t="s">
         <v>17</v>
@@ -11286,7 +11286,7 @@
         <v>51</v>
       </c>
       <c r="K218" s="7">
-        <v>305</v>
+        <v>586</v>
       </c>
       <c r="L218" s="5" t="s">
         <v>17</v>
@@ -11324,7 +11324,7 @@
         <v>55</v>
       </c>
       <c r="K219" s="8">
-        <v>756</v>
+        <v>792</v>
       </c>
       <c r="L219" s="5" t="s">
         <v>17</v>
@@ -11362,7 +11362,7 @@
         <v>59</v>
       </c>
       <c r="K220" s="7">
-        <v>163</v>
+        <v>820</v>
       </c>
       <c r="L220" s="5" t="s">
         <v>17</v>
@@ -11400,7 +11400,7 @@
         <v>51</v>
       </c>
       <c r="K221" s="8">
-        <v>487</v>
+        <v>155</v>
       </c>
       <c r="L221" s="5" t="s">
         <v>17</v>
@@ -11438,7 +11438,7 @@
         <v>55</v>
       </c>
       <c r="K222" s="7">
-        <v>175</v>
+        <v>851</v>
       </c>
       <c r="L222" s="5" t="s">
         <v>17</v>
@@ -11476,7 +11476,7 @@
         <v>59</v>
       </c>
       <c r="K223" s="8">
-        <v>621</v>
+        <v>301</v>
       </c>
       <c r="L223" s="5" t="s">
         <v>17</v>
@@ -11514,7 +11514,7 @@
         <v>51</v>
       </c>
       <c r="K224" s="7">
-        <v>357</v>
+        <v>641</v>
       </c>
       <c r="L224" s="5" t="s">
         <v>17</v>
@@ -11552,7 +11552,7 @@
         <v>55</v>
       </c>
       <c r="K225" s="8">
-        <v>452</v>
+        <v>219</v>
       </c>
       <c r="L225" s="5" t="s">
         <v>17</v>
@@ -11590,7 +11590,7 @@
         <v>59</v>
       </c>
       <c r="K226" s="7">
-        <v>750</v>
+        <v>132</v>
       </c>
       <c r="L226" s="5" t="s">
         <v>17</v>
@@ -11628,7 +11628,7 @@
         <v>51</v>
       </c>
       <c r="K227" s="8">
-        <v>824</v>
+        <v>397</v>
       </c>
       <c r="L227" s="5" t="s">
         <v>17</v>
@@ -11666,7 +11666,7 @@
         <v>55</v>
       </c>
       <c r="K228" s="7">
-        <v>141</v>
+        <v>689</v>
       </c>
       <c r="L228" s="5" t="s">
         <v>17</v>
@@ -11704,7 +11704,7 @@
         <v>59</v>
       </c>
       <c r="K229" s="8">
-        <v>963</v>
+        <v>216</v>
       </c>
       <c r="L229" s="5" t="s">
         <v>17</v>
@@ -11742,7 +11742,7 @@
         <v>51</v>
       </c>
       <c r="K230" s="7">
-        <v>451</v>
+        <v>424</v>
       </c>
       <c r="L230" s="5" t="s">
         <v>17</v>
@@ -11780,7 +11780,7 @@
         <v>55</v>
       </c>
       <c r="K231" s="8">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="L231" s="5" t="s">
         <v>17</v>
@@ -11818,7 +11818,7 @@
         <v>59</v>
       </c>
       <c r="K232" s="7">
-        <v>767</v>
+        <v>263</v>
       </c>
       <c r="L232" s="5" t="s">
         <v>17</v>
@@ -11856,7 +11856,7 @@
         <v>51</v>
       </c>
       <c r="K233" s="8">
-        <v>549</v>
+        <v>419</v>
       </c>
       <c r="L233" s="5" t="s">
         <v>17</v>
@@ -11894,7 +11894,7 @@
         <v>55</v>
       </c>
       <c r="K234" s="7">
-        <v>739</v>
+        <v>662</v>
       </c>
       <c r="L234" s="5" t="s">
         <v>17</v>
@@ -11932,7 +11932,7 @@
         <v>59</v>
       </c>
       <c r="K235" s="8">
-        <v>944</v>
+        <v>291</v>
       </c>
       <c r="L235" s="5" t="s">
         <v>17</v>
@@ -11970,7 +11970,7 @@
         <v>51</v>
       </c>
       <c r="K236" s="7">
-        <v>892</v>
+        <v>346</v>
       </c>
       <c r="L236" s="5" t="s">
         <v>17</v>
@@ -12008,7 +12008,7 @@
         <v>55</v>
       </c>
       <c r="K237" s="8">
-        <v>814</v>
+        <v>601</v>
       </c>
       <c r="L237" s="5" t="s">
         <v>17</v>
@@ -12046,7 +12046,7 @@
         <v>59</v>
       </c>
       <c r="K238" s="7">
-        <v>560</v>
+        <v>477</v>
       </c>
       <c r="L238" s="5" t="s">
         <v>17</v>
@@ -12084,7 +12084,7 @@
         <v>51</v>
       </c>
       <c r="K239" s="8">
-        <v>839</v>
+        <v>197</v>
       </c>
       <c r="L239" s="5" t="s">
         <v>17</v>
@@ -12122,7 +12122,7 @@
         <v>55</v>
       </c>
       <c r="K240" s="7">
-        <v>962</v>
+        <v>297</v>
       </c>
       <c r="L240" s="5" t="s">
         <v>17</v>
@@ -12160,7 +12160,7 @@
         <v>59</v>
       </c>
       <c r="K241" s="8">
-        <v>186</v>
+        <v>795</v>
       </c>
       <c r="L241" s="5" t="s">
         <v>17</v>
@@ -12198,7 +12198,7 @@
         <v>51</v>
       </c>
       <c r="K242" s="7">
-        <v>375</v>
+        <v>197</v>
       </c>
       <c r="L242" s="5" t="s">
         <v>17</v>
@@ -12236,7 +12236,7 @@
         <v>55</v>
       </c>
       <c r="K243" s="8">
-        <v>934</v>
+        <v>944</v>
       </c>
       <c r="L243" s="5" t="s">
         <v>17</v>
@@ -12274,7 +12274,7 @@
         <v>59</v>
       </c>
       <c r="K244" s="7">
-        <v>542</v>
+        <v>711</v>
       </c>
       <c r="L244" s="5" t="s">
         <v>17</v>
@@ -12312,7 +12312,7 @@
         <v>51</v>
       </c>
       <c r="K245" s="8">
-        <v>538</v>
+        <v>187</v>
       </c>
       <c r="L245" s="5" t="s">
         <v>17</v>
@@ -12350,7 +12350,7 @@
         <v>55</v>
       </c>
       <c r="K246" s="7">
-        <v>708</v>
+        <v>808</v>
       </c>
       <c r="L246" s="5" t="s">
         <v>17</v>
@@ -12388,7 +12388,7 @@
         <v>59</v>
       </c>
       <c r="K247" s="8">
-        <v>749</v>
+        <v>210</v>
       </c>
       <c r="L247" s="9" t="s">
         <v>142</v>
@@ -12426,7 +12426,7 @@
         <v>51</v>
       </c>
       <c r="K248" s="7">
-        <v>575</v>
+        <v>323</v>
       </c>
       <c r="L248" s="5" t="s">
         <v>17</v>
@@ -12464,7 +12464,7 @@
         <v>55</v>
       </c>
       <c r="K249" s="8">
-        <v>674</v>
+        <v>149</v>
       </c>
       <c r="L249" s="5" t="s">
         <v>17</v>
@@ -12502,7 +12502,7 @@
         <v>59</v>
       </c>
       <c r="K250" s="7">
-        <v>418</v>
+        <v>508</v>
       </c>
       <c r="L250" s="5" t="s">
         <v>17</v>
@@ -12540,7 +12540,7 @@
         <v>51</v>
       </c>
       <c r="K251" s="8">
-        <v>732</v>
+        <v>491</v>
       </c>
       <c r="L251" s="5" t="s">
         <v>17</v>
@@ -12578,7 +12578,7 @@
         <v>55</v>
       </c>
       <c r="K252" s="7">
-        <v>782</v>
+        <v>676</v>
       </c>
       <c r="L252" s="5" t="s">
         <v>17</v>
@@ -12616,7 +12616,7 @@
         <v>59</v>
       </c>
       <c r="K253" s="8">
-        <v>160</v>
+        <v>536</v>
       </c>
       <c r="L253" s="5" t="s">
         <v>17</v>
@@ -12654,7 +12654,7 @@
         <v>51</v>
       </c>
       <c r="K254" s="7">
-        <v>701</v>
+        <v>533</v>
       </c>
       <c r="L254" s="5" t="s">
         <v>17</v>
@@ -12692,7 +12692,7 @@
         <v>55</v>
       </c>
       <c r="K255" s="8">
-        <v>239</v>
+        <v>528</v>
       </c>
       <c r="L255" s="5" t="s">
         <v>17</v>
@@ -12730,7 +12730,7 @@
         <v>59</v>
       </c>
       <c r="K256" s="7">
-        <v>700</v>
+        <v>296</v>
       </c>
       <c r="L256" s="5" t="s">
         <v>17</v>
@@ -12768,7 +12768,7 @@
         <v>51</v>
       </c>
       <c r="K257" s="8">
-        <v>673</v>
+        <v>156</v>
       </c>
       <c r="L257" s="5" t="s">
         <v>17</v>
@@ -12806,7 +12806,7 @@
         <v>55</v>
       </c>
       <c r="K258" s="7">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="L258" s="5" t="s">
         <v>17</v>
@@ -12844,7 +12844,7 @@
         <v>59</v>
       </c>
       <c r="K259" s="8">
-        <v>859</v>
+        <v>563</v>
       </c>
       <c r="L259" s="5" t="s">
         <v>17</v>
@@ -12882,7 +12882,7 @@
         <v>51</v>
       </c>
       <c r="K260" s="7">
-        <v>217</v>
+        <v>713</v>
       </c>
       <c r="L260" s="5" t="s">
         <v>17</v>
@@ -12920,7 +12920,7 @@
         <v>55</v>
       </c>
       <c r="K261" s="8">
-        <v>290</v>
+        <v>566</v>
       </c>
       <c r="L261" s="5" t="s">
         <v>17</v>
@@ -12958,7 +12958,7 @@
         <v>59</v>
       </c>
       <c r="K262" s="7">
-        <v>332</v>
+        <v>404</v>
       </c>
       <c r="L262" s="5" t="s">
         <v>17</v>
@@ -12996,7 +12996,7 @@
         <v>51</v>
       </c>
       <c r="K263" s="8">
-        <v>582</v>
+        <v>374</v>
       </c>
       <c r="L263" s="5" t="s">
         <v>17</v>
@@ -13034,7 +13034,7 @@
         <v>55</v>
       </c>
       <c r="K264" s="7">
-        <v>374</v>
+        <v>276</v>
       </c>
       <c r="L264" s="5" t="s">
         <v>17</v>
@@ -13072,7 +13072,7 @@
         <v>59</v>
       </c>
       <c r="K265" s="8">
-        <v>486</v>
+        <v>282</v>
       </c>
       <c r="L265" s="5" t="s">
         <v>17</v>
@@ -13110,7 +13110,7 @@
         <v>51</v>
       </c>
       <c r="K266" s="7">
-        <v>350</v>
+        <v>539</v>
       </c>
       <c r="L266" s="5" t="s">
         <v>17</v>
@@ -13148,7 +13148,7 @@
         <v>55</v>
       </c>
       <c r="K267" s="8">
-        <v>596</v>
+        <v>189</v>
       </c>
       <c r="L267" s="5" t="s">
         <v>17</v>
@@ -13186,7 +13186,7 @@
         <v>59</v>
       </c>
       <c r="K268" s="7">
-        <v>590</v>
+        <v>566</v>
       </c>
       <c r="L268" s="10" t="s">
         <v>244</v>
@@ -13224,7 +13224,7 @@
         <v>51</v>
       </c>
       <c r="K269" s="8">
-        <v>855</v>
+        <v>750</v>
       </c>
       <c r="L269" s="5" t="s">
         <v>17</v>
@@ -13262,7 +13262,7 @@
         <v>55</v>
       </c>
       <c r="K270" s="7">
-        <v>415</v>
+        <v>609</v>
       </c>
       <c r="L270" s="5" t="s">
         <v>17</v>
@@ -13300,7 +13300,7 @@
         <v>59</v>
       </c>
       <c r="K271" s="8">
-        <v>137</v>
+        <v>308</v>
       </c>
       <c r="L271" s="5" t="s">
         <v>17</v>
@@ -13338,7 +13338,7 @@
         <v>51</v>
       </c>
       <c r="K272" s="7">
-        <v>836</v>
+        <v>848</v>
       </c>
       <c r="L272" s="5" t="s">
         <v>17</v>
@@ -13376,7 +13376,7 @@
         <v>55</v>
       </c>
       <c r="K273" s="8">
-        <v>746</v>
+        <v>716</v>
       </c>
       <c r="L273" s="5" t="s">
         <v>17</v>
@@ -13414,7 +13414,7 @@
         <v>59</v>
       </c>
       <c r="K274" s="7">
-        <v>667</v>
+        <v>716</v>
       </c>
       <c r="L274" s="5" t="s">
         <v>17</v>
@@ -13452,7 +13452,7 @@
         <v>51</v>
       </c>
       <c r="K275" s="8">
-        <v>392</v>
+        <v>727</v>
       </c>
       <c r="L275" s="5" t="s">
         <v>17</v>
@@ -13490,7 +13490,7 @@
         <v>55</v>
       </c>
       <c r="K276" s="7">
-        <v>214</v>
+        <v>622</v>
       </c>
       <c r="L276" s="5" t="s">
         <v>17</v>
@@ -13528,7 +13528,7 @@
         <v>59</v>
       </c>
       <c r="K277" s="8">
-        <v>307</v>
+        <v>693</v>
       </c>
       <c r="L277" s="5" t="s">
         <v>17</v>
@@ -13566,7 +13566,7 @@
         <v>51</v>
       </c>
       <c r="K278" s="7">
-        <v>619</v>
+        <v>449</v>
       </c>
       <c r="L278" s="5" t="s">
         <v>17</v>
@@ -13604,7 +13604,7 @@
         <v>55</v>
       </c>
       <c r="K279" s="8">
-        <v>674</v>
+        <v>128</v>
       </c>
       <c r="L279" s="5" t="s">
         <v>17</v>
@@ -13642,7 +13642,7 @@
         <v>59</v>
       </c>
       <c r="K280" s="7">
-        <v>409</v>
+        <v>771</v>
       </c>
       <c r="L280" s="5" t="s">
         <v>17</v>
@@ -13680,7 +13680,7 @@
         <v>51</v>
       </c>
       <c r="K281" s="8">
-        <v>181</v>
+        <v>148</v>
       </c>
       <c r="L281" s="5" t="s">
         <v>17</v>
@@ -13718,7 +13718,7 @@
         <v>55</v>
       </c>
       <c r="K282" s="7">
-        <v>652</v>
+        <v>547</v>
       </c>
       <c r="L282" s="5" t="s">
         <v>17</v>
@@ -13756,7 +13756,7 @@
         <v>59</v>
       </c>
       <c r="K283" s="8">
-        <v>218</v>
+        <v>508</v>
       </c>
       <c r="L283" s="5" t="s">
         <v>17</v>
@@ -13794,7 +13794,7 @@
         <v>51</v>
       </c>
       <c r="K284" s="7">
-        <v>477</v>
+        <v>708</v>
       </c>
       <c r="L284" s="5" t="s">
         <v>17</v>
@@ -13832,7 +13832,7 @@
         <v>55</v>
       </c>
       <c r="K285" s="8">
-        <v>483</v>
+        <v>855</v>
       </c>
       <c r="L285" s="5" t="s">
         <v>17</v>
@@ -13870,7 +13870,7 @@
         <v>59</v>
       </c>
       <c r="K286" s="7">
-        <v>722</v>
+        <v>350</v>
       </c>
       <c r="L286" s="5" t="s">
         <v>17</v>
@@ -13908,7 +13908,7 @@
         <v>51</v>
       </c>
       <c r="K287" s="8">
-        <v>490</v>
+        <v>449</v>
       </c>
       <c r="L287" s="5" t="s">
         <v>17</v>
@@ -13946,7 +13946,7 @@
         <v>55</v>
       </c>
       <c r="K288" s="7">
-        <v>857</v>
+        <v>425</v>
       </c>
       <c r="L288" s="9" t="s">
         <v>142</v>
@@ -13984,7 +13984,7 @@
         <v>59</v>
       </c>
       <c r="K289" s="8">
-        <v>814</v>
+        <v>656</v>
       </c>
       <c r="L289" s="5" t="s">
         <v>17</v>
@@ -14022,7 +14022,7 @@
         <v>51</v>
       </c>
       <c r="K290" s="7">
-        <v>536</v>
+        <v>774</v>
       </c>
       <c r="L290" s="5" t="s">
         <v>17</v>
@@ -14060,7 +14060,7 @@
         <v>55</v>
       </c>
       <c r="K291" s="8">
-        <v>701</v>
+        <v>857</v>
       </c>
       <c r="L291" s="5" t="s">
         <v>17</v>
@@ -14098,7 +14098,7 @@
         <v>59</v>
       </c>
       <c r="K292" s="7">
-        <v>392</v>
+        <v>197</v>
       </c>
       <c r="L292" s="5" t="s">
         <v>17</v>
@@ -14136,7 +14136,7 @@
         <v>51</v>
       </c>
       <c r="K293" s="8">
-        <v>636</v>
+        <v>253</v>
       </c>
       <c r="L293" s="5" t="s">
         <v>17</v>
@@ -14174,7 +14174,7 @@
         <v>55</v>
       </c>
       <c r="K294" s="7">
-        <v>775</v>
+        <v>465</v>
       </c>
       <c r="L294" s="5" t="s">
         <v>17</v>
@@ -14212,7 +14212,7 @@
         <v>59</v>
       </c>
       <c r="K295" s="8">
-        <v>580</v>
+        <v>443</v>
       </c>
       <c r="L295" s="5" t="s">
         <v>17</v>
@@ -14250,7 +14250,7 @@
         <v>51</v>
       </c>
       <c r="K296" s="7">
-        <v>667</v>
+        <v>300</v>
       </c>
       <c r="L296" s="5" t="s">
         <v>17</v>
@@ -14288,7 +14288,7 @@
         <v>55</v>
       </c>
       <c r="K297" s="8">
-        <v>905</v>
+        <v>581</v>
       </c>
       <c r="L297" s="5" t="s">
         <v>17</v>
@@ -14326,7 +14326,7 @@
         <v>59</v>
       </c>
       <c r="K298" s="7">
-        <v>669</v>
+        <v>144</v>
       </c>
       <c r="L298" s="5" t="s">
         <v>17</v>
@@ -14364,7 +14364,7 @@
         <v>51</v>
       </c>
       <c r="K299" s="8">
-        <v>844</v>
+        <v>646</v>
       </c>
       <c r="L299" s="5" t="s">
         <v>17</v>
@@ -14402,7 +14402,7 @@
         <v>55</v>
       </c>
       <c r="K300" s="7">
-        <v>269</v>
+        <v>187</v>
       </c>
       <c r="L300" s="5" t="s">
         <v>17</v>
@@ -14440,7 +14440,7 @@
         <v>59</v>
       </c>
       <c r="K301" s="8">
-        <v>831</v>
+        <v>885</v>
       </c>
       <c r="L301" s="5" t="s">
         <v>17</v>
@@ -14478,7 +14478,7 @@
         <v>51</v>
       </c>
       <c r="K302" s="7">
-        <v>806</v>
+        <v>565</v>
       </c>
       <c r="L302" s="5" t="s">
         <v>17</v>
@@ -14516,7 +14516,7 @@
         <v>55</v>
       </c>
       <c r="K303" s="8">
-        <v>543</v>
+        <v>408</v>
       </c>
       <c r="L303" s="5" t="s">
         <v>17</v>
@@ -14554,7 +14554,7 @@
         <v>59</v>
       </c>
       <c r="K304" s="7">
-        <v>744</v>
+        <v>414</v>
       </c>
       <c r="L304" s="5" t="s">
         <v>17</v>
@@ -14592,7 +14592,7 @@
         <v>51</v>
       </c>
       <c r="K305" s="8">
-        <v>899</v>
+        <v>288</v>
       </c>
       <c r="L305" s="5" t="s">
         <v>17</v>
@@ -14630,7 +14630,7 @@
         <v>55</v>
       </c>
       <c r="K306" s="7">
-        <v>611</v>
+        <v>276</v>
       </c>
       <c r="L306" s="5" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
docs(qa): update master QA dashboard and test reports across all domains
</commit_message>
<xml_diff>
--- a/frontend/selenium-tests/live-selenium-report.xlsx
+++ b/frontend/selenium-tests/live-selenium-report.xlsx
@@ -38,7 +38,7 @@
     <t>Execution Timestamp</t>
   </si>
   <si>
-    <t>24/7/2026, 7:03:56 pm</t>
+    <t>24/7/2026, 7:25:02 pm</t>
   </si>
   <si>
     <t>Browser Environment</t>
@@ -3078,7 +3078,7 @@
         <v>51</v>
       </c>
       <c r="K2" s="7">
-        <v>357</v>
+        <v>251</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>17</v>
@@ -3116,7 +3116,7 @@
         <v>55</v>
       </c>
       <c r="K3" s="8">
-        <v>912</v>
+        <v>500</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>17</v>
@@ -3154,7 +3154,7 @@
         <v>59</v>
       </c>
       <c r="K4" s="7">
-        <v>447</v>
+        <v>597</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>17</v>
@@ -3192,7 +3192,7 @@
         <v>51</v>
       </c>
       <c r="K5" s="8">
-        <v>143</v>
+        <v>961</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>17</v>
@@ -3230,7 +3230,7 @@
         <v>55</v>
       </c>
       <c r="K6" s="7">
-        <v>660</v>
+        <v>806</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>17</v>
@@ -3268,7 +3268,7 @@
         <v>59</v>
       </c>
       <c r="K7" s="8">
-        <v>165</v>
+        <v>436</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>17</v>
@@ -3306,7 +3306,7 @@
         <v>51</v>
       </c>
       <c r="K8" s="7">
-        <v>246</v>
+        <v>147</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>17</v>
@@ -3344,7 +3344,7 @@
         <v>55</v>
       </c>
       <c r="K9" s="8">
-        <v>915</v>
+        <v>956</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>17</v>
@@ -3382,7 +3382,7 @@
         <v>59</v>
       </c>
       <c r="K10" s="7">
-        <v>698</v>
+        <v>144</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>17</v>
@@ -3420,7 +3420,7 @@
         <v>51</v>
       </c>
       <c r="K11" s="8">
-        <v>612</v>
+        <v>432</v>
       </c>
       <c r="L11" s="5" t="s">
         <v>17</v>
@@ -3458,7 +3458,7 @@
         <v>55</v>
       </c>
       <c r="K12" s="7">
-        <v>885</v>
+        <v>888</v>
       </c>
       <c r="L12" s="5" t="s">
         <v>17</v>
@@ -3496,7 +3496,7 @@
         <v>59</v>
       </c>
       <c r="K13" s="8">
-        <v>500</v>
+        <v>480</v>
       </c>
       <c r="L13" s="5" t="s">
         <v>17</v>
@@ -3534,7 +3534,7 @@
         <v>51</v>
       </c>
       <c r="K14" s="7">
-        <v>304</v>
+        <v>961</v>
       </c>
       <c r="L14" s="5" t="s">
         <v>17</v>
@@ -3572,7 +3572,7 @@
         <v>55</v>
       </c>
       <c r="K15" s="8">
-        <v>413</v>
+        <v>354</v>
       </c>
       <c r="L15" s="5" t="s">
         <v>17</v>
@@ -3610,7 +3610,7 @@
         <v>59</v>
       </c>
       <c r="K16" s="7">
-        <v>420</v>
+        <v>783</v>
       </c>
       <c r="L16" s="5" t="s">
         <v>17</v>
@@ -3648,7 +3648,7 @@
         <v>51</v>
       </c>
       <c r="K17" s="8">
-        <v>828</v>
+        <v>943</v>
       </c>
       <c r="L17" s="5" t="s">
         <v>17</v>
@@ -3686,7 +3686,7 @@
         <v>55</v>
       </c>
       <c r="K18" s="7">
-        <v>319</v>
+        <v>840</v>
       </c>
       <c r="L18" s="5" t="s">
         <v>17</v>
@@ -3724,7 +3724,7 @@
         <v>59</v>
       </c>
       <c r="K19" s="8">
-        <v>493</v>
+        <v>444</v>
       </c>
       <c r="L19" s="5" t="s">
         <v>17</v>
@@ -3762,7 +3762,7 @@
         <v>51</v>
       </c>
       <c r="K20" s="7">
-        <v>479</v>
+        <v>167</v>
       </c>
       <c r="L20" s="5" t="s">
         <v>17</v>
@@ -3800,7 +3800,7 @@
         <v>55</v>
       </c>
       <c r="K21" s="8">
-        <v>447</v>
+        <v>722</v>
       </c>
       <c r="L21" s="5" t="s">
         <v>17</v>
@@ -3838,7 +3838,7 @@
         <v>59</v>
       </c>
       <c r="K22" s="7">
-        <v>821</v>
+        <v>897</v>
       </c>
       <c r="L22" s="5" t="s">
         <v>17</v>
@@ -3876,7 +3876,7 @@
         <v>51</v>
       </c>
       <c r="K23" s="8">
-        <v>658</v>
+        <v>229</v>
       </c>
       <c r="L23" s="5" t="s">
         <v>17</v>
@@ -3914,7 +3914,7 @@
         <v>55</v>
       </c>
       <c r="K24" s="7">
-        <v>314</v>
+        <v>218</v>
       </c>
       <c r="L24" s="5" t="s">
         <v>17</v>
@@ -3952,7 +3952,7 @@
         <v>59</v>
       </c>
       <c r="K25" s="8">
-        <v>808</v>
+        <v>280</v>
       </c>
       <c r="L25" s="5" t="s">
         <v>17</v>
@@ -3990,7 +3990,7 @@
         <v>51</v>
       </c>
       <c r="K26" s="7">
-        <v>842</v>
+        <v>456</v>
       </c>
       <c r="L26" s="5" t="s">
         <v>17</v>
@@ -4028,7 +4028,7 @@
         <v>55</v>
       </c>
       <c r="K27" s="8">
-        <v>725</v>
+        <v>346</v>
       </c>
       <c r="L27" s="5" t="s">
         <v>17</v>
@@ -4066,7 +4066,7 @@
         <v>59</v>
       </c>
       <c r="K28" s="7">
-        <v>902</v>
+        <v>851</v>
       </c>
       <c r="L28" s="5" t="s">
         <v>17</v>
@@ -4104,7 +4104,7 @@
         <v>51</v>
       </c>
       <c r="K29" s="8">
-        <v>303</v>
+        <v>429</v>
       </c>
       <c r="L29" s="5" t="s">
         <v>17</v>
@@ -4142,7 +4142,7 @@
         <v>55</v>
       </c>
       <c r="K30" s="7">
-        <v>828</v>
+        <v>537</v>
       </c>
       <c r="L30" s="5" t="s">
         <v>17</v>
@@ -4180,7 +4180,7 @@
         <v>59</v>
       </c>
       <c r="K31" s="8">
-        <v>618</v>
+        <v>309</v>
       </c>
       <c r="L31" s="5" t="s">
         <v>17</v>
@@ -4218,7 +4218,7 @@
         <v>51</v>
       </c>
       <c r="K32" s="7">
-        <v>439</v>
+        <v>578</v>
       </c>
       <c r="L32" s="5" t="s">
         <v>17</v>
@@ -4256,7 +4256,7 @@
         <v>55</v>
       </c>
       <c r="K33" s="8">
-        <v>260</v>
+        <v>714</v>
       </c>
       <c r="L33" s="5" t="s">
         <v>17</v>
@@ -4294,7 +4294,7 @@
         <v>59</v>
       </c>
       <c r="K34" s="7">
-        <v>908</v>
+        <v>577</v>
       </c>
       <c r="L34" s="5" t="s">
         <v>17</v>
@@ -4332,7 +4332,7 @@
         <v>51</v>
       </c>
       <c r="K35" s="8">
-        <v>829</v>
+        <v>413</v>
       </c>
       <c r="L35" s="5" t="s">
         <v>17</v>
@@ -4370,7 +4370,7 @@
         <v>55</v>
       </c>
       <c r="K36" s="7">
-        <v>687</v>
+        <v>905</v>
       </c>
       <c r="L36" s="5" t="s">
         <v>17</v>
@@ -4408,7 +4408,7 @@
         <v>59</v>
       </c>
       <c r="K37" s="8">
-        <v>188</v>
+        <v>263</v>
       </c>
       <c r="L37" s="5" t="s">
         <v>17</v>
@@ -4446,7 +4446,7 @@
         <v>51</v>
       </c>
       <c r="K38" s="7">
-        <v>952</v>
+        <v>276</v>
       </c>
       <c r="L38" s="5" t="s">
         <v>17</v>
@@ -4484,7 +4484,7 @@
         <v>55</v>
       </c>
       <c r="K39" s="8">
-        <v>623</v>
+        <v>562</v>
       </c>
       <c r="L39" s="5" t="s">
         <v>17</v>
@@ -4522,7 +4522,7 @@
         <v>59</v>
       </c>
       <c r="K40" s="7">
-        <v>550</v>
+        <v>876</v>
       </c>
       <c r="L40" s="5" t="s">
         <v>17</v>
@@ -4560,7 +4560,7 @@
         <v>51</v>
       </c>
       <c r="K41" s="8">
-        <v>424</v>
+        <v>233</v>
       </c>
       <c r="L41" s="5" t="s">
         <v>17</v>
@@ -4598,7 +4598,7 @@
         <v>55</v>
       </c>
       <c r="K42" s="7">
-        <v>592</v>
+        <v>534</v>
       </c>
       <c r="L42" s="9" t="s">
         <v>142</v>
@@ -4636,7 +4636,7 @@
         <v>59</v>
       </c>
       <c r="K43" s="8">
-        <v>167</v>
+        <v>337</v>
       </c>
       <c r="L43" s="5" t="s">
         <v>17</v>
@@ -4674,7 +4674,7 @@
         <v>51</v>
       </c>
       <c r="K44" s="7">
-        <v>527</v>
+        <v>299</v>
       </c>
       <c r="L44" s="5" t="s">
         <v>17</v>
@@ -4712,7 +4712,7 @@
         <v>55</v>
       </c>
       <c r="K45" s="8">
-        <v>822</v>
+        <v>941</v>
       </c>
       <c r="L45" s="5" t="s">
         <v>17</v>
@@ -4750,7 +4750,7 @@
         <v>59</v>
       </c>
       <c r="K46" s="7">
-        <v>331</v>
+        <v>277</v>
       </c>
       <c r="L46" s="5" t="s">
         <v>17</v>
@@ -4788,7 +4788,7 @@
         <v>51</v>
       </c>
       <c r="K47" s="8">
-        <v>127</v>
+        <v>502</v>
       </c>
       <c r="L47" s="5" t="s">
         <v>17</v>
@@ -4826,7 +4826,7 @@
         <v>55</v>
       </c>
       <c r="K48" s="7">
-        <v>158</v>
+        <v>123</v>
       </c>
       <c r="L48" s="5" t="s">
         <v>17</v>
@@ -4864,7 +4864,7 @@
         <v>59</v>
       </c>
       <c r="K49" s="8">
-        <v>152</v>
+        <v>676</v>
       </c>
       <c r="L49" s="5" t="s">
         <v>17</v>
@@ -4940,7 +4940,7 @@
         <v>55</v>
       </c>
       <c r="K51" s="8">
-        <v>935</v>
+        <v>557</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>17</v>
@@ -4978,7 +4978,7 @@
         <v>59</v>
       </c>
       <c r="K52" s="7">
-        <v>422</v>
+        <v>553</v>
       </c>
       <c r="L52" s="5" t="s">
         <v>17</v>
@@ -5016,7 +5016,7 @@
         <v>51</v>
       </c>
       <c r="K53" s="8">
-        <v>959</v>
+        <v>458</v>
       </c>
       <c r="L53" s="5" t="s">
         <v>17</v>
@@ -5054,7 +5054,7 @@
         <v>55</v>
       </c>
       <c r="K54" s="7">
-        <v>894</v>
+        <v>230</v>
       </c>
       <c r="L54" s="5" t="s">
         <v>17</v>
@@ -5092,7 +5092,7 @@
         <v>59</v>
       </c>
       <c r="K55" s="8">
-        <v>352</v>
+        <v>699</v>
       </c>
       <c r="L55" s="5" t="s">
         <v>17</v>
@@ -5130,7 +5130,7 @@
         <v>51</v>
       </c>
       <c r="K56" s="7">
-        <v>822</v>
+        <v>632</v>
       </c>
       <c r="L56" s="5" t="s">
         <v>17</v>
@@ -5168,7 +5168,7 @@
         <v>55</v>
       </c>
       <c r="K57" s="8">
-        <v>160</v>
+        <v>575</v>
       </c>
       <c r="L57" s="5" t="s">
         <v>17</v>
@@ -5206,7 +5206,7 @@
         <v>59</v>
       </c>
       <c r="K58" s="7">
-        <v>787</v>
+        <v>234</v>
       </c>
       <c r="L58" s="5" t="s">
         <v>17</v>
@@ -5244,7 +5244,7 @@
         <v>51</v>
       </c>
       <c r="K59" s="8">
-        <v>773</v>
+        <v>137</v>
       </c>
       <c r="L59" s="5" t="s">
         <v>17</v>
@@ -5282,7 +5282,7 @@
         <v>55</v>
       </c>
       <c r="K60" s="7">
-        <v>496</v>
+        <v>436</v>
       </c>
       <c r="L60" s="5" t="s">
         <v>17</v>
@@ -5320,7 +5320,7 @@
         <v>59</v>
       </c>
       <c r="K61" s="8">
-        <v>820</v>
+        <v>530</v>
       </c>
       <c r="L61" s="5" t="s">
         <v>17</v>
@@ -5358,7 +5358,7 @@
         <v>51</v>
       </c>
       <c r="K62" s="7">
-        <v>524</v>
+        <v>670</v>
       </c>
       <c r="L62" s="5" t="s">
         <v>17</v>
@@ -5396,7 +5396,7 @@
         <v>55</v>
       </c>
       <c r="K63" s="8">
-        <v>712</v>
+        <v>151</v>
       </c>
       <c r="L63" s="5" t="s">
         <v>17</v>
@@ -5434,7 +5434,7 @@
         <v>59</v>
       </c>
       <c r="K64" s="7">
-        <v>801</v>
+        <v>541</v>
       </c>
       <c r="L64" s="5" t="s">
         <v>17</v>
@@ -5472,7 +5472,7 @@
         <v>51</v>
       </c>
       <c r="K65" s="8">
-        <v>844</v>
+        <v>456</v>
       </c>
       <c r="L65" s="5" t="s">
         <v>17</v>
@@ -5510,7 +5510,7 @@
         <v>55</v>
       </c>
       <c r="K66" s="7">
-        <v>409</v>
+        <v>647</v>
       </c>
       <c r="L66" s="5" t="s">
         <v>17</v>
@@ -5548,7 +5548,7 @@
         <v>59</v>
       </c>
       <c r="K67" s="8">
-        <v>123</v>
+        <v>282</v>
       </c>
       <c r="L67" s="5" t="s">
         <v>17</v>
@@ -5586,7 +5586,7 @@
         <v>51</v>
       </c>
       <c r="K68" s="7">
-        <v>514</v>
+        <v>852</v>
       </c>
       <c r="L68" s="5" t="s">
         <v>17</v>
@@ -5624,7 +5624,7 @@
         <v>55</v>
       </c>
       <c r="K69" s="8">
-        <v>198</v>
+        <v>399</v>
       </c>
       <c r="L69" s="5" t="s">
         <v>17</v>
@@ -5662,7 +5662,7 @@
         <v>59</v>
       </c>
       <c r="K70" s="7">
-        <v>956</v>
+        <v>750</v>
       </c>
       <c r="L70" s="5" t="s">
         <v>17</v>
@@ -5700,7 +5700,7 @@
         <v>51</v>
       </c>
       <c r="K71" s="8">
-        <v>244</v>
+        <v>750</v>
       </c>
       <c r="L71" s="5" t="s">
         <v>17</v>
@@ -5738,7 +5738,7 @@
         <v>55</v>
       </c>
       <c r="K72" s="7">
-        <v>191</v>
+        <v>146</v>
       </c>
       <c r="L72" s="5" t="s">
         <v>17</v>
@@ -5776,7 +5776,7 @@
         <v>59</v>
       </c>
       <c r="K73" s="8">
-        <v>582</v>
+        <v>678</v>
       </c>
       <c r="L73" s="5" t="s">
         <v>17</v>
@@ -5814,7 +5814,7 @@
         <v>51</v>
       </c>
       <c r="K74" s="7">
-        <v>922</v>
+        <v>361</v>
       </c>
       <c r="L74" s="5" t="s">
         <v>17</v>
@@ -5852,7 +5852,7 @@
         <v>55</v>
       </c>
       <c r="K75" s="8">
-        <v>406</v>
+        <v>340</v>
       </c>
       <c r="L75" s="5" t="s">
         <v>17</v>
@@ -5890,7 +5890,7 @@
         <v>59</v>
       </c>
       <c r="K76" s="7">
-        <v>826</v>
+        <v>595</v>
       </c>
       <c r="L76" s="5" t="s">
         <v>17</v>
@@ -5966,7 +5966,7 @@
         <v>55</v>
       </c>
       <c r="K78" s="7">
-        <v>203</v>
+        <v>174</v>
       </c>
       <c r="L78" s="5" t="s">
         <v>17</v>
@@ -6004,7 +6004,7 @@
         <v>59</v>
       </c>
       <c r="K79" s="8">
-        <v>708</v>
+        <v>415</v>
       </c>
       <c r="L79" s="5" t="s">
         <v>17</v>
@@ -6042,7 +6042,7 @@
         <v>51</v>
       </c>
       <c r="K80" s="7">
-        <v>693</v>
+        <v>642</v>
       </c>
       <c r="L80" s="5" t="s">
         <v>17</v>
@@ -6080,7 +6080,7 @@
         <v>55</v>
       </c>
       <c r="K81" s="8">
-        <v>341</v>
+        <v>192</v>
       </c>
       <c r="L81" s="5" t="s">
         <v>17</v>
@@ -6118,7 +6118,7 @@
         <v>59</v>
       </c>
       <c r="K82" s="7">
-        <v>799</v>
+        <v>865</v>
       </c>
       <c r="L82" s="5" t="s">
         <v>17</v>
@@ -6156,7 +6156,7 @@
         <v>51</v>
       </c>
       <c r="K83" s="8">
-        <v>762</v>
+        <v>405</v>
       </c>
       <c r="L83" s="9" t="s">
         <v>142</v>
@@ -6194,7 +6194,7 @@
         <v>55</v>
       </c>
       <c r="K84" s="7">
-        <v>181</v>
+        <v>572</v>
       </c>
       <c r="L84" s="5" t="s">
         <v>17</v>
@@ -6232,7 +6232,7 @@
         <v>59</v>
       </c>
       <c r="K85" s="8">
-        <v>571</v>
+        <v>212</v>
       </c>
       <c r="L85" s="5" t="s">
         <v>17</v>
@@ -6270,7 +6270,7 @@
         <v>51</v>
       </c>
       <c r="K86" s="7">
-        <v>887</v>
+        <v>341</v>
       </c>
       <c r="L86" s="5" t="s">
         <v>17</v>
@@ -6308,7 +6308,7 @@
         <v>55</v>
       </c>
       <c r="K87" s="8">
-        <v>675</v>
+        <v>217</v>
       </c>
       <c r="L87" s="5" t="s">
         <v>17</v>
@@ -6346,7 +6346,7 @@
         <v>59</v>
       </c>
       <c r="K88" s="7">
-        <v>253</v>
+        <v>162</v>
       </c>
       <c r="L88" s="5" t="s">
         <v>17</v>
@@ -6384,7 +6384,7 @@
         <v>51</v>
       </c>
       <c r="K89" s="8">
-        <v>916</v>
+        <v>887</v>
       </c>
       <c r="L89" s="5" t="s">
         <v>17</v>
@@ -6422,7 +6422,7 @@
         <v>55</v>
       </c>
       <c r="K90" s="7">
-        <v>238</v>
+        <v>155</v>
       </c>
       <c r="L90" s="10" t="s">
         <v>244</v>
@@ -6460,7 +6460,7 @@
         <v>59</v>
       </c>
       <c r="K91" s="8">
-        <v>213</v>
+        <v>964</v>
       </c>
       <c r="L91" s="5" t="s">
         <v>17</v>
@@ -6498,7 +6498,7 @@
         <v>51</v>
       </c>
       <c r="K92" s="7">
-        <v>734</v>
+        <v>787</v>
       </c>
       <c r="L92" s="5" t="s">
         <v>17</v>
@@ -6536,7 +6536,7 @@
         <v>55</v>
       </c>
       <c r="K93" s="8">
-        <v>642</v>
+        <v>846</v>
       </c>
       <c r="L93" s="5" t="s">
         <v>17</v>
@@ -6574,7 +6574,7 @@
         <v>59</v>
       </c>
       <c r="K94" s="7">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="L94" s="5" t="s">
         <v>17</v>
@@ -6612,7 +6612,7 @@
         <v>51</v>
       </c>
       <c r="K95" s="8">
-        <v>624</v>
+        <v>781</v>
       </c>
       <c r="L95" s="5" t="s">
         <v>17</v>
@@ -6650,7 +6650,7 @@
         <v>55</v>
       </c>
       <c r="K96" s="7">
-        <v>548</v>
+        <v>967</v>
       </c>
       <c r="L96" s="5" t="s">
         <v>17</v>
@@ -6688,7 +6688,7 @@
         <v>59</v>
       </c>
       <c r="K97" s="8">
-        <v>682</v>
+        <v>451</v>
       </c>
       <c r="L97" s="5" t="s">
         <v>17</v>
@@ -6726,7 +6726,7 @@
         <v>51</v>
       </c>
       <c r="K98" s="7">
-        <v>184</v>
+        <v>339</v>
       </c>
       <c r="L98" s="5" t="s">
         <v>17</v>
@@ -6764,7 +6764,7 @@
         <v>55</v>
       </c>
       <c r="K99" s="8">
-        <v>126</v>
+        <v>883</v>
       </c>
       <c r="L99" s="5" t="s">
         <v>17</v>
@@ -6802,7 +6802,7 @@
         <v>59</v>
       </c>
       <c r="K100" s="7">
-        <v>510</v>
+        <v>710</v>
       </c>
       <c r="L100" s="5" t="s">
         <v>17</v>
@@ -6840,7 +6840,7 @@
         <v>51</v>
       </c>
       <c r="K101" s="8">
-        <v>281</v>
+        <v>188</v>
       </c>
       <c r="L101" s="5" t="s">
         <v>17</v>
@@ -6878,7 +6878,7 @@
         <v>55</v>
       </c>
       <c r="K102" s="7">
-        <v>805</v>
+        <v>125</v>
       </c>
       <c r="L102" s="5" t="s">
         <v>17</v>
@@ -6916,7 +6916,7 @@
         <v>59</v>
       </c>
       <c r="K103" s="8">
-        <v>432</v>
+        <v>617</v>
       </c>
       <c r="L103" s="5" t="s">
         <v>17</v>
@@ -6954,7 +6954,7 @@
         <v>51</v>
       </c>
       <c r="K104" s="7">
-        <v>573</v>
+        <v>587</v>
       </c>
       <c r="L104" s="5" t="s">
         <v>17</v>
@@ -6992,7 +6992,7 @@
         <v>55</v>
       </c>
       <c r="K105" s="8">
-        <v>930</v>
+        <v>790</v>
       </c>
       <c r="L105" s="5" t="s">
         <v>17</v>
@@ -7030,7 +7030,7 @@
         <v>59</v>
       </c>
       <c r="K106" s="7">
-        <v>879</v>
+        <v>511</v>
       </c>
       <c r="L106" s="5" t="s">
         <v>17</v>
@@ -7068,7 +7068,7 @@
         <v>51</v>
       </c>
       <c r="K107" s="8">
-        <v>954</v>
+        <v>278</v>
       </c>
       <c r="L107" s="5" t="s">
         <v>17</v>
@@ -7106,7 +7106,7 @@
         <v>55</v>
       </c>
       <c r="K108" s="7">
-        <v>895</v>
+        <v>253</v>
       </c>
       <c r="L108" s="5" t="s">
         <v>17</v>
@@ -7144,7 +7144,7 @@
         <v>59</v>
       </c>
       <c r="K109" s="8">
-        <v>404</v>
+        <v>772</v>
       </c>
       <c r="L109" s="5" t="s">
         <v>17</v>
@@ -7182,7 +7182,7 @@
         <v>51</v>
       </c>
       <c r="K110" s="7">
-        <v>166</v>
+        <v>659</v>
       </c>
       <c r="L110" s="5" t="s">
         <v>17</v>
@@ -7220,7 +7220,7 @@
         <v>55</v>
       </c>
       <c r="K111" s="8">
-        <v>478</v>
+        <v>545</v>
       </c>
       <c r="L111" s="5" t="s">
         <v>17</v>
@@ -7258,7 +7258,7 @@
         <v>59</v>
       </c>
       <c r="K112" s="7">
-        <v>907</v>
+        <v>630</v>
       </c>
       <c r="L112" s="5" t="s">
         <v>17</v>
@@ -7296,7 +7296,7 @@
         <v>51</v>
       </c>
       <c r="K113" s="8">
-        <v>456</v>
+        <v>385</v>
       </c>
       <c r="L113" s="5" t="s">
         <v>17</v>
@@ -7334,7 +7334,7 @@
         <v>55</v>
       </c>
       <c r="K114" s="7">
-        <v>910</v>
+        <v>317</v>
       </c>
       <c r="L114" s="5" t="s">
         <v>17</v>
@@ -7372,7 +7372,7 @@
         <v>59</v>
       </c>
       <c r="K115" s="8">
-        <v>755</v>
+        <v>721</v>
       </c>
       <c r="L115" s="5" t="s">
         <v>17</v>
@@ -7410,7 +7410,7 @@
         <v>51</v>
       </c>
       <c r="K116" s="7">
-        <v>193</v>
+        <v>406</v>
       </c>
       <c r="L116" s="5" t="s">
         <v>17</v>
@@ -7448,7 +7448,7 @@
         <v>55</v>
       </c>
       <c r="K117" s="8">
-        <v>490</v>
+        <v>906</v>
       </c>
       <c r="L117" s="5" t="s">
         <v>17</v>
@@ -7486,7 +7486,7 @@
         <v>59</v>
       </c>
       <c r="K118" s="7">
-        <v>343</v>
+        <v>814</v>
       </c>
       <c r="L118" s="5" t="s">
         <v>17</v>
@@ -7524,7 +7524,7 @@
         <v>51</v>
       </c>
       <c r="K119" s="8">
-        <v>133</v>
+        <v>291</v>
       </c>
       <c r="L119" s="5" t="s">
         <v>17</v>
@@ -7562,7 +7562,7 @@
         <v>55</v>
       </c>
       <c r="K120" s="7">
-        <v>734</v>
+        <v>379</v>
       </c>
       <c r="L120" s="5" t="s">
         <v>17</v>
@@ -7600,7 +7600,7 @@
         <v>59</v>
       </c>
       <c r="K121" s="8">
-        <v>533</v>
+        <v>156</v>
       </c>
       <c r="L121" s="5" t="s">
         <v>17</v>
@@ -7638,7 +7638,7 @@
         <v>51</v>
       </c>
       <c r="K122" s="7">
-        <v>501</v>
+        <v>693</v>
       </c>
       <c r="L122" s="5" t="s">
         <v>17</v>
@@ -7676,7 +7676,7 @@
         <v>55</v>
       </c>
       <c r="K123" s="8">
-        <v>225</v>
+        <v>470</v>
       </c>
       <c r="L123" s="5" t="s">
         <v>17</v>
@@ -7714,7 +7714,7 @@
         <v>59</v>
       </c>
       <c r="K124" s="7">
-        <v>809</v>
+        <v>829</v>
       </c>
       <c r="L124" s="9" t="s">
         <v>142</v>
@@ -7752,7 +7752,7 @@
         <v>51</v>
       </c>
       <c r="K125" s="8">
-        <v>268</v>
+        <v>592</v>
       </c>
       <c r="L125" s="5" t="s">
         <v>17</v>
@@ -7790,7 +7790,7 @@
         <v>55</v>
       </c>
       <c r="K126" s="7">
-        <v>766</v>
+        <v>510</v>
       </c>
       <c r="L126" s="5" t="s">
         <v>17</v>
@@ -7828,7 +7828,7 @@
         <v>59</v>
       </c>
       <c r="K127" s="8">
-        <v>763</v>
+        <v>891</v>
       </c>
       <c r="L127" s="5" t="s">
         <v>17</v>
@@ -7866,7 +7866,7 @@
         <v>51</v>
       </c>
       <c r="K128" s="7">
-        <v>281</v>
+        <v>424</v>
       </c>
       <c r="L128" s="5" t="s">
         <v>17</v>
@@ -7904,7 +7904,7 @@
         <v>55</v>
       </c>
       <c r="K129" s="8">
-        <v>907</v>
+        <v>217</v>
       </c>
       <c r="L129" s="5" t="s">
         <v>17</v>
@@ -7942,7 +7942,7 @@
         <v>59</v>
       </c>
       <c r="K130" s="7">
-        <v>598</v>
+        <v>821</v>
       </c>
       <c r="L130" s="5" t="s">
         <v>17</v>
@@ -7980,7 +7980,7 @@
         <v>51</v>
       </c>
       <c r="K131" s="8">
-        <v>609</v>
+        <v>305</v>
       </c>
       <c r="L131" s="5" t="s">
         <v>17</v>
@@ -8018,7 +8018,7 @@
         <v>55</v>
       </c>
       <c r="K132" s="7">
-        <v>936</v>
+        <v>751</v>
       </c>
       <c r="L132" s="5" t="s">
         <v>17</v>
@@ -8056,7 +8056,7 @@
         <v>59</v>
       </c>
       <c r="K133" s="8">
-        <v>668</v>
+        <v>398</v>
       </c>
       <c r="L133" s="5" t="s">
         <v>17</v>
@@ -8094,7 +8094,7 @@
         <v>51</v>
       </c>
       <c r="K134" s="7">
-        <v>572</v>
+        <v>722</v>
       </c>
       <c r="L134" s="5" t="s">
         <v>17</v>
@@ -8132,7 +8132,7 @@
         <v>55</v>
       </c>
       <c r="K135" s="8">
-        <v>189</v>
+        <v>693</v>
       </c>
       <c r="L135" s="5" t="s">
         <v>17</v>
@@ -8170,7 +8170,7 @@
         <v>59</v>
       </c>
       <c r="K136" s="7">
-        <v>357</v>
+        <v>198</v>
       </c>
       <c r="L136" s="5" t="s">
         <v>17</v>
@@ -8208,7 +8208,7 @@
         <v>51</v>
       </c>
       <c r="K137" s="8">
-        <v>428</v>
+        <v>329</v>
       </c>
       <c r="L137" s="5" t="s">
         <v>17</v>
@@ -8246,7 +8246,7 @@
         <v>55</v>
       </c>
       <c r="K138" s="7">
-        <v>668</v>
+        <v>389</v>
       </c>
       <c r="L138" s="5" t="s">
         <v>17</v>
@@ -8284,7 +8284,7 @@
         <v>59</v>
       </c>
       <c r="K139" s="8">
-        <v>688</v>
+        <v>367</v>
       </c>
       <c r="L139" s="5" t="s">
         <v>17</v>
@@ -8322,7 +8322,7 @@
         <v>51</v>
       </c>
       <c r="K140" s="7">
-        <v>356</v>
+        <v>247</v>
       </c>
       <c r="L140" s="5" t="s">
         <v>17</v>
@@ -8360,7 +8360,7 @@
         <v>55</v>
       </c>
       <c r="K141" s="8">
-        <v>700</v>
+        <v>349</v>
       </c>
       <c r="L141" s="5" t="s">
         <v>17</v>
@@ -8398,7 +8398,7 @@
         <v>59</v>
       </c>
       <c r="K142" s="7">
-        <v>669</v>
+        <v>240</v>
       </c>
       <c r="L142" s="5" t="s">
         <v>17</v>
@@ -8436,7 +8436,7 @@
         <v>51</v>
       </c>
       <c r="K143" s="8">
-        <v>366</v>
+        <v>857</v>
       </c>
       <c r="L143" s="5" t="s">
         <v>17</v>
@@ -8474,7 +8474,7 @@
         <v>55</v>
       </c>
       <c r="K144" s="7">
-        <v>244</v>
+        <v>535</v>
       </c>
       <c r="L144" s="5" t="s">
         <v>17</v>
@@ -8512,7 +8512,7 @@
         <v>59</v>
       </c>
       <c r="K145" s="8">
-        <v>350</v>
+        <v>840</v>
       </c>
       <c r="L145" s="5" t="s">
         <v>17</v>
@@ -8550,7 +8550,7 @@
         <v>51</v>
       </c>
       <c r="K146" s="7">
-        <v>666</v>
+        <v>965</v>
       </c>
       <c r="L146" s="5" t="s">
         <v>17</v>
@@ -8588,7 +8588,7 @@
         <v>55</v>
       </c>
       <c r="K147" s="8">
-        <v>585</v>
+        <v>254</v>
       </c>
       <c r="L147" s="5" t="s">
         <v>17</v>
@@ -8626,7 +8626,7 @@
         <v>59</v>
       </c>
       <c r="K148" s="7">
-        <v>131</v>
+        <v>195</v>
       </c>
       <c r="L148" s="5" t="s">
         <v>17</v>
@@ -8664,7 +8664,7 @@
         <v>51</v>
       </c>
       <c r="K149" s="8">
-        <v>240</v>
+        <v>445</v>
       </c>
       <c r="L149" s="5" t="s">
         <v>17</v>
@@ -8702,7 +8702,7 @@
         <v>55</v>
       </c>
       <c r="K150" s="7">
-        <v>890</v>
+        <v>222</v>
       </c>
       <c r="L150" s="5" t="s">
         <v>17</v>
@@ -8740,7 +8740,7 @@
         <v>59</v>
       </c>
       <c r="K151" s="8">
-        <v>576</v>
+        <v>675</v>
       </c>
       <c r="L151" s="5" t="s">
         <v>17</v>
@@ -8778,7 +8778,7 @@
         <v>51</v>
       </c>
       <c r="K152" s="7">
-        <v>189</v>
+        <v>217</v>
       </c>
       <c r="L152" s="5" t="s">
         <v>17</v>
@@ -8816,7 +8816,7 @@
         <v>55</v>
       </c>
       <c r="K153" s="8">
-        <v>171</v>
+        <v>900</v>
       </c>
       <c r="L153" s="5" t="s">
         <v>17</v>
@@ -8854,7 +8854,7 @@
         <v>59</v>
       </c>
       <c r="K154" s="7">
-        <v>820</v>
+        <v>899</v>
       </c>
       <c r="L154" s="5" t="s">
         <v>17</v>
@@ -8892,7 +8892,7 @@
         <v>51</v>
       </c>
       <c r="K155" s="8">
-        <v>497</v>
+        <v>205</v>
       </c>
       <c r="L155" s="5" t="s">
         <v>17</v>
@@ -8930,7 +8930,7 @@
         <v>55</v>
       </c>
       <c r="K156" s="7">
-        <v>122</v>
+        <v>383</v>
       </c>
       <c r="L156" s="5" t="s">
         <v>17</v>
@@ -8968,7 +8968,7 @@
         <v>59</v>
       </c>
       <c r="K157" s="8">
-        <v>279</v>
+        <v>541</v>
       </c>
       <c r="L157" s="5" t="s">
         <v>17</v>
@@ -9006,7 +9006,7 @@
         <v>51</v>
       </c>
       <c r="K158" s="7">
-        <v>230</v>
+        <v>793</v>
       </c>
       <c r="L158" s="5" t="s">
         <v>17</v>
@@ -9044,7 +9044,7 @@
         <v>55</v>
       </c>
       <c r="K159" s="8">
-        <v>484</v>
+        <v>754</v>
       </c>
       <c r="L159" s="5" t="s">
         <v>17</v>
@@ -9082,7 +9082,7 @@
         <v>59</v>
       </c>
       <c r="K160" s="7">
-        <v>255</v>
+        <v>304</v>
       </c>
       <c r="L160" s="5" t="s">
         <v>17</v>
@@ -9120,7 +9120,7 @@
         <v>51</v>
       </c>
       <c r="K161" s="8">
-        <v>790</v>
+        <v>388</v>
       </c>
       <c r="L161" s="5" t="s">
         <v>17</v>
@@ -9158,7 +9158,7 @@
         <v>55</v>
       </c>
       <c r="K162" s="7">
-        <v>540</v>
+        <v>737</v>
       </c>
       <c r="L162" s="5" t="s">
         <v>17</v>
@@ -9196,7 +9196,7 @@
         <v>59</v>
       </c>
       <c r="K163" s="8">
-        <v>762</v>
+        <v>334</v>
       </c>
       <c r="L163" s="5" t="s">
         <v>17</v>
@@ -9234,7 +9234,7 @@
         <v>51</v>
       </c>
       <c r="K164" s="7">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="L164" s="5" t="s">
         <v>17</v>
@@ -9272,7 +9272,7 @@
         <v>55</v>
       </c>
       <c r="K165" s="8">
-        <v>264</v>
+        <v>709</v>
       </c>
       <c r="L165" s="9" t="s">
         <v>142</v>
@@ -9310,7 +9310,7 @@
         <v>59</v>
       </c>
       <c r="K166" s="7">
-        <v>969</v>
+        <v>410</v>
       </c>
       <c r="L166" s="5" t="s">
         <v>17</v>
@@ -9348,7 +9348,7 @@
         <v>51</v>
       </c>
       <c r="K167" s="8">
-        <v>318</v>
+        <v>720</v>
       </c>
       <c r="L167" s="5" t="s">
         <v>17</v>
@@ -9386,7 +9386,7 @@
         <v>55</v>
       </c>
       <c r="K168" s="7">
-        <v>741</v>
+        <v>417</v>
       </c>
       <c r="L168" s="5" t="s">
         <v>17</v>
@@ -9424,7 +9424,7 @@
         <v>59</v>
       </c>
       <c r="K169" s="8">
-        <v>731</v>
+        <v>282</v>
       </c>
       <c r="L169" s="5" t="s">
         <v>17</v>
@@ -9462,7 +9462,7 @@
         <v>51</v>
       </c>
       <c r="K170" s="7">
-        <v>284</v>
+        <v>673</v>
       </c>
       <c r="L170" s="5" t="s">
         <v>17</v>
@@ -9500,7 +9500,7 @@
         <v>55</v>
       </c>
       <c r="K171" s="8">
-        <v>444</v>
+        <v>544</v>
       </c>
       <c r="L171" s="5" t="s">
         <v>17</v>
@@ -9538,7 +9538,7 @@
         <v>59</v>
       </c>
       <c r="K172" s="7">
-        <v>724</v>
+        <v>631</v>
       </c>
       <c r="L172" s="5" t="s">
         <v>17</v>
@@ -9576,7 +9576,7 @@
         <v>51</v>
       </c>
       <c r="K173" s="8">
-        <v>751</v>
+        <v>204</v>
       </c>
       <c r="L173" s="5" t="s">
         <v>17</v>
@@ -9614,7 +9614,7 @@
         <v>55</v>
       </c>
       <c r="K174" s="7">
-        <v>490</v>
+        <v>627</v>
       </c>
       <c r="L174" s="5" t="s">
         <v>17</v>
@@ -9652,7 +9652,7 @@
         <v>59</v>
       </c>
       <c r="K175" s="8">
-        <v>266</v>
+        <v>625</v>
       </c>
       <c r="L175" s="5" t="s">
         <v>17</v>
@@ -9690,7 +9690,7 @@
         <v>51</v>
       </c>
       <c r="K176" s="7">
-        <v>480</v>
+        <v>383</v>
       </c>
       <c r="L176" s="5" t="s">
         <v>17</v>
@@ -9728,7 +9728,7 @@
         <v>55</v>
       </c>
       <c r="K177" s="8">
-        <v>472</v>
+        <v>429</v>
       </c>
       <c r="L177" s="5" t="s">
         <v>17</v>
@@ -9766,7 +9766,7 @@
         <v>59</v>
       </c>
       <c r="K178" s="7">
-        <v>621</v>
+        <v>685</v>
       </c>
       <c r="L178" s="5" t="s">
         <v>17</v>
@@ -9804,7 +9804,7 @@
         <v>51</v>
       </c>
       <c r="K179" s="8">
-        <v>949</v>
+        <v>805</v>
       </c>
       <c r="L179" s="10" t="s">
         <v>244</v>
@@ -9842,7 +9842,7 @@
         <v>55</v>
       </c>
       <c r="K180" s="7">
-        <v>315</v>
+        <v>884</v>
       </c>
       <c r="L180" s="5" t="s">
         <v>17</v>
@@ -9880,7 +9880,7 @@
         <v>59</v>
       </c>
       <c r="K181" s="8">
-        <v>284</v>
+        <v>713</v>
       </c>
       <c r="L181" s="5" t="s">
         <v>17</v>
@@ -9918,7 +9918,7 @@
         <v>51</v>
       </c>
       <c r="K182" s="7">
-        <v>874</v>
+        <v>541</v>
       </c>
       <c r="L182" s="5" t="s">
         <v>17</v>
@@ -9956,7 +9956,7 @@
         <v>55</v>
       </c>
       <c r="K183" s="8">
-        <v>220</v>
+        <v>827</v>
       </c>
       <c r="L183" s="5" t="s">
         <v>17</v>
@@ -9994,7 +9994,7 @@
         <v>59</v>
       </c>
       <c r="K184" s="7">
-        <v>483</v>
+        <v>336</v>
       </c>
       <c r="L184" s="5" t="s">
         <v>17</v>
@@ -10032,7 +10032,7 @@
         <v>51</v>
       </c>
       <c r="K185" s="8">
-        <v>961</v>
+        <v>681</v>
       </c>
       <c r="L185" s="5" t="s">
         <v>17</v>
@@ -10070,7 +10070,7 @@
         <v>55</v>
       </c>
       <c r="K186" s="7">
-        <v>123</v>
+        <v>544</v>
       </c>
       <c r="L186" s="5" t="s">
         <v>17</v>
@@ -10108,7 +10108,7 @@
         <v>59</v>
       </c>
       <c r="K187" s="8">
-        <v>728</v>
+        <v>266</v>
       </c>
       <c r="L187" s="5" t="s">
         <v>17</v>
@@ -10146,7 +10146,7 @@
         <v>51</v>
       </c>
       <c r="K188" s="7">
-        <v>775</v>
+        <v>455</v>
       </c>
       <c r="L188" s="5" t="s">
         <v>17</v>
@@ -10184,7 +10184,7 @@
         <v>55</v>
       </c>
       <c r="K189" s="8">
-        <v>838</v>
+        <v>658</v>
       </c>
       <c r="L189" s="5" t="s">
         <v>17</v>
@@ -10222,7 +10222,7 @@
         <v>59</v>
       </c>
       <c r="K190" s="7">
-        <v>153</v>
+        <v>587</v>
       </c>
       <c r="L190" s="5" t="s">
         <v>17</v>
@@ -10260,7 +10260,7 @@
         <v>51</v>
       </c>
       <c r="K191" s="8">
-        <v>120</v>
+        <v>758</v>
       </c>
       <c r="L191" s="5" t="s">
         <v>17</v>
@@ -10298,7 +10298,7 @@
         <v>55</v>
       </c>
       <c r="K192" s="7">
-        <v>207</v>
+        <v>658</v>
       </c>
       <c r="L192" s="5" t="s">
         <v>17</v>
@@ -10336,7 +10336,7 @@
         <v>59</v>
       </c>
       <c r="K193" s="8">
-        <v>414</v>
+        <v>138</v>
       </c>
       <c r="L193" s="5" t="s">
         <v>17</v>
@@ -10374,7 +10374,7 @@
         <v>51</v>
       </c>
       <c r="K194" s="7">
-        <v>855</v>
+        <v>541</v>
       </c>
       <c r="L194" s="5" t="s">
         <v>17</v>
@@ -10412,7 +10412,7 @@
         <v>55</v>
       </c>
       <c r="K195" s="8">
-        <v>831</v>
+        <v>272</v>
       </c>
       <c r="L195" s="5" t="s">
         <v>17</v>
@@ -10450,7 +10450,7 @@
         <v>59</v>
       </c>
       <c r="K196" s="7">
-        <v>740</v>
+        <v>842</v>
       </c>
       <c r="L196" s="5" t="s">
         <v>17</v>
@@ -10488,7 +10488,7 @@
         <v>51</v>
       </c>
       <c r="K197" s="8">
-        <v>265</v>
+        <v>148</v>
       </c>
       <c r="L197" s="5" t="s">
         <v>17</v>
@@ -10526,7 +10526,7 @@
         <v>55</v>
       </c>
       <c r="K198" s="7">
-        <v>420</v>
+        <v>184</v>
       </c>
       <c r="L198" s="5" t="s">
         <v>17</v>
@@ -10564,7 +10564,7 @@
         <v>59</v>
       </c>
       <c r="K199" s="8">
-        <v>834</v>
+        <v>807</v>
       </c>
       <c r="L199" s="5" t="s">
         <v>17</v>
@@ -10602,7 +10602,7 @@
         <v>51</v>
       </c>
       <c r="K200" s="7">
-        <v>168</v>
+        <v>748</v>
       </c>
       <c r="L200" s="5" t="s">
         <v>17</v>
@@ -10640,7 +10640,7 @@
         <v>55</v>
       </c>
       <c r="K201" s="8">
-        <v>512</v>
+        <v>681</v>
       </c>
       <c r="L201" s="5" t="s">
         <v>17</v>
@@ -10678,7 +10678,7 @@
         <v>59</v>
       </c>
       <c r="K202" s="7">
-        <v>681</v>
+        <v>889</v>
       </c>
       <c r="L202" s="5" t="s">
         <v>17</v>
@@ -10716,7 +10716,7 @@
         <v>51</v>
       </c>
       <c r="K203" s="8">
-        <v>147</v>
+        <v>786</v>
       </c>
       <c r="L203" s="5" t="s">
         <v>17</v>
@@ -10754,7 +10754,7 @@
         <v>55</v>
       </c>
       <c r="K204" s="7">
-        <v>304</v>
+        <v>423</v>
       </c>
       <c r="L204" s="5" t="s">
         <v>17</v>
@@ -10792,7 +10792,7 @@
         <v>59</v>
       </c>
       <c r="K205" s="8">
-        <v>739</v>
+        <v>332</v>
       </c>
       <c r="L205" s="5" t="s">
         <v>17</v>
@@ -10830,7 +10830,7 @@
         <v>51</v>
       </c>
       <c r="K206" s="7">
-        <v>293</v>
+        <v>910</v>
       </c>
       <c r="L206" s="9" t="s">
         <v>142</v>
@@ -10868,7 +10868,7 @@
         <v>55</v>
       </c>
       <c r="K207" s="8">
-        <v>747</v>
+        <v>656</v>
       </c>
       <c r="L207" s="5" t="s">
         <v>17</v>
@@ -10906,7 +10906,7 @@
         <v>59</v>
       </c>
       <c r="K208" s="7">
-        <v>849</v>
+        <v>499</v>
       </c>
       <c r="L208" s="5" t="s">
         <v>17</v>
@@ -10944,7 +10944,7 @@
         <v>51</v>
       </c>
       <c r="K209" s="8">
-        <v>309</v>
+        <v>685</v>
       </c>
       <c r="L209" s="5" t="s">
         <v>17</v>
@@ -10982,7 +10982,7 @@
         <v>55</v>
       </c>
       <c r="K210" s="7">
-        <v>528</v>
+        <v>500</v>
       </c>
       <c r="L210" s="5" t="s">
         <v>17</v>
@@ -11020,7 +11020,7 @@
         <v>59</v>
       </c>
       <c r="K211" s="8">
-        <v>230</v>
+        <v>345</v>
       </c>
       <c r="L211" s="5" t="s">
         <v>17</v>
@@ -11058,7 +11058,7 @@
         <v>51</v>
       </c>
       <c r="K212" s="7">
-        <v>836</v>
+        <v>155</v>
       </c>
       <c r="L212" s="5" t="s">
         <v>17</v>
@@ -11096,7 +11096,7 @@
         <v>55</v>
       </c>
       <c r="K213" s="8">
-        <v>550</v>
+        <v>712</v>
       </c>
       <c r="L213" s="5" t="s">
         <v>17</v>
@@ -11134,7 +11134,7 @@
         <v>59</v>
       </c>
       <c r="K214" s="7">
-        <v>855</v>
+        <v>869</v>
       </c>
       <c r="L214" s="5" t="s">
         <v>17</v>
@@ -11172,7 +11172,7 @@
         <v>51</v>
       </c>
       <c r="K215" s="8">
-        <v>156</v>
+        <v>355</v>
       </c>
       <c r="L215" s="5" t="s">
         <v>17</v>
@@ -11210,7 +11210,7 @@
         <v>55</v>
       </c>
       <c r="K216" s="7">
-        <v>254</v>
+        <v>462</v>
       </c>
       <c r="L216" s="5" t="s">
         <v>17</v>
@@ -11248,7 +11248,7 @@
         <v>59</v>
       </c>
       <c r="K217" s="8">
-        <v>805</v>
+        <v>707</v>
       </c>
       <c r="L217" s="5" t="s">
         <v>17</v>
@@ -11286,7 +11286,7 @@
         <v>51</v>
       </c>
       <c r="K218" s="7">
-        <v>586</v>
+        <v>639</v>
       </c>
       <c r="L218" s="5" t="s">
         <v>17</v>
@@ -11324,7 +11324,7 @@
         <v>55</v>
       </c>
       <c r="K219" s="8">
-        <v>792</v>
+        <v>908</v>
       </c>
       <c r="L219" s="5" t="s">
         <v>17</v>
@@ -11362,7 +11362,7 @@
         <v>59</v>
       </c>
       <c r="K220" s="7">
-        <v>820</v>
+        <v>709</v>
       </c>
       <c r="L220" s="5" t="s">
         <v>17</v>
@@ -11400,7 +11400,7 @@
         <v>51</v>
       </c>
       <c r="K221" s="8">
-        <v>155</v>
+        <v>271</v>
       </c>
       <c r="L221" s="5" t="s">
         <v>17</v>
@@ -11438,7 +11438,7 @@
         <v>55</v>
       </c>
       <c r="K222" s="7">
-        <v>851</v>
+        <v>682</v>
       </c>
       <c r="L222" s="5" t="s">
         <v>17</v>
@@ -11476,7 +11476,7 @@
         <v>59</v>
       </c>
       <c r="K223" s="8">
-        <v>301</v>
+        <v>963</v>
       </c>
       <c r="L223" s="5" t="s">
         <v>17</v>
@@ -11514,7 +11514,7 @@
         <v>51</v>
       </c>
       <c r="K224" s="7">
-        <v>641</v>
+        <v>192</v>
       </c>
       <c r="L224" s="5" t="s">
         <v>17</v>
@@ -11552,7 +11552,7 @@
         <v>55</v>
       </c>
       <c r="K225" s="8">
-        <v>219</v>
+        <v>956</v>
       </c>
       <c r="L225" s="5" t="s">
         <v>17</v>
@@ -11590,7 +11590,7 @@
         <v>59</v>
       </c>
       <c r="K226" s="7">
-        <v>132</v>
+        <v>552</v>
       </c>
       <c r="L226" s="5" t="s">
         <v>17</v>
@@ -11628,7 +11628,7 @@
         <v>51</v>
       </c>
       <c r="K227" s="8">
-        <v>397</v>
+        <v>874</v>
       </c>
       <c r="L227" s="5" t="s">
         <v>17</v>
@@ -11666,7 +11666,7 @@
         <v>55</v>
       </c>
       <c r="K228" s="7">
-        <v>689</v>
+        <v>194</v>
       </c>
       <c r="L228" s="5" t="s">
         <v>17</v>
@@ -11704,7 +11704,7 @@
         <v>59</v>
       </c>
       <c r="K229" s="8">
-        <v>216</v>
+        <v>646</v>
       </c>
       <c r="L229" s="5" t="s">
         <v>17</v>
@@ -11742,7 +11742,7 @@
         <v>51</v>
       </c>
       <c r="K230" s="7">
-        <v>424</v>
+        <v>845</v>
       </c>
       <c r="L230" s="5" t="s">
         <v>17</v>
@@ -11780,7 +11780,7 @@
         <v>55</v>
       </c>
       <c r="K231" s="8">
-        <v>549</v>
+        <v>825</v>
       </c>
       <c r="L231" s="5" t="s">
         <v>17</v>
@@ -11818,7 +11818,7 @@
         <v>59</v>
       </c>
       <c r="K232" s="7">
-        <v>263</v>
+        <v>446</v>
       </c>
       <c r="L232" s="5" t="s">
         <v>17</v>
@@ -11856,7 +11856,7 @@
         <v>51</v>
       </c>
       <c r="K233" s="8">
-        <v>419</v>
+        <v>199</v>
       </c>
       <c r="L233" s="5" t="s">
         <v>17</v>
@@ -11894,7 +11894,7 @@
         <v>55</v>
       </c>
       <c r="K234" s="7">
-        <v>662</v>
+        <v>767</v>
       </c>
       <c r="L234" s="5" t="s">
         <v>17</v>
@@ -11932,7 +11932,7 @@
         <v>59</v>
       </c>
       <c r="K235" s="8">
-        <v>291</v>
+        <v>885</v>
       </c>
       <c r="L235" s="5" t="s">
         <v>17</v>
@@ -11970,7 +11970,7 @@
         <v>51</v>
       </c>
       <c r="K236" s="7">
-        <v>346</v>
+        <v>160</v>
       </c>
       <c r="L236" s="5" t="s">
         <v>17</v>
@@ -12008,7 +12008,7 @@
         <v>55</v>
       </c>
       <c r="K237" s="8">
-        <v>601</v>
+        <v>674</v>
       </c>
       <c r="L237" s="5" t="s">
         <v>17</v>
@@ -12046,7 +12046,7 @@
         <v>59</v>
       </c>
       <c r="K238" s="7">
-        <v>477</v>
+        <v>854</v>
       </c>
       <c r="L238" s="5" t="s">
         <v>17</v>
@@ -12084,7 +12084,7 @@
         <v>51</v>
       </c>
       <c r="K239" s="8">
-        <v>197</v>
+        <v>261</v>
       </c>
       <c r="L239" s="5" t="s">
         <v>17</v>
@@ -12122,7 +12122,7 @@
         <v>55</v>
       </c>
       <c r="K240" s="7">
-        <v>297</v>
+        <v>888</v>
       </c>
       <c r="L240" s="5" t="s">
         <v>17</v>
@@ -12160,7 +12160,7 @@
         <v>59</v>
       </c>
       <c r="K241" s="8">
-        <v>795</v>
+        <v>375</v>
       </c>
       <c r="L241" s="5" t="s">
         <v>17</v>
@@ -12198,7 +12198,7 @@
         <v>51</v>
       </c>
       <c r="K242" s="7">
-        <v>197</v>
+        <v>488</v>
       </c>
       <c r="L242" s="5" t="s">
         <v>17</v>
@@ -12236,7 +12236,7 @@
         <v>55</v>
       </c>
       <c r="K243" s="8">
-        <v>944</v>
+        <v>871</v>
       </c>
       <c r="L243" s="5" t="s">
         <v>17</v>
@@ -12274,7 +12274,7 @@
         <v>59</v>
       </c>
       <c r="K244" s="7">
-        <v>711</v>
+        <v>377</v>
       </c>
       <c r="L244" s="5" t="s">
         <v>17</v>
@@ -12312,7 +12312,7 @@
         <v>51</v>
       </c>
       <c r="K245" s="8">
-        <v>187</v>
+        <v>150</v>
       </c>
       <c r="L245" s="5" t="s">
         <v>17</v>
@@ -12350,7 +12350,7 @@
         <v>55</v>
       </c>
       <c r="K246" s="7">
-        <v>808</v>
+        <v>311</v>
       </c>
       <c r="L246" s="5" t="s">
         <v>17</v>
@@ -12388,7 +12388,7 @@
         <v>59</v>
       </c>
       <c r="K247" s="8">
-        <v>210</v>
+        <v>495</v>
       </c>
       <c r="L247" s="9" t="s">
         <v>142</v>
@@ -12426,7 +12426,7 @@
         <v>51</v>
       </c>
       <c r="K248" s="7">
-        <v>323</v>
+        <v>248</v>
       </c>
       <c r="L248" s="5" t="s">
         <v>17</v>
@@ -12464,7 +12464,7 @@
         <v>55</v>
       </c>
       <c r="K249" s="8">
-        <v>149</v>
+        <v>327</v>
       </c>
       <c r="L249" s="5" t="s">
         <v>17</v>
@@ -12502,7 +12502,7 @@
         <v>59</v>
       </c>
       <c r="K250" s="7">
-        <v>508</v>
+        <v>189</v>
       </c>
       <c r="L250" s="5" t="s">
         <v>17</v>
@@ -12540,7 +12540,7 @@
         <v>51</v>
       </c>
       <c r="K251" s="8">
-        <v>491</v>
+        <v>723</v>
       </c>
       <c r="L251" s="5" t="s">
         <v>17</v>
@@ -12578,7 +12578,7 @@
         <v>55</v>
       </c>
       <c r="K252" s="7">
-        <v>676</v>
+        <v>543</v>
       </c>
       <c r="L252" s="5" t="s">
         <v>17</v>
@@ -12616,7 +12616,7 @@
         <v>59</v>
       </c>
       <c r="K253" s="8">
-        <v>536</v>
+        <v>298</v>
       </c>
       <c r="L253" s="5" t="s">
         <v>17</v>
@@ -12654,7 +12654,7 @@
         <v>51</v>
       </c>
       <c r="K254" s="7">
-        <v>533</v>
+        <v>273</v>
       </c>
       <c r="L254" s="5" t="s">
         <v>17</v>
@@ -12692,7 +12692,7 @@
         <v>55</v>
       </c>
       <c r="K255" s="8">
-        <v>528</v>
+        <v>634</v>
       </c>
       <c r="L255" s="5" t="s">
         <v>17</v>
@@ -12730,7 +12730,7 @@
         <v>59</v>
       </c>
       <c r="K256" s="7">
-        <v>296</v>
+        <v>721</v>
       </c>
       <c r="L256" s="5" t="s">
         <v>17</v>
@@ -12768,7 +12768,7 @@
         <v>51</v>
       </c>
       <c r="K257" s="8">
-        <v>156</v>
+        <v>594</v>
       </c>
       <c r="L257" s="5" t="s">
         <v>17</v>
@@ -12806,7 +12806,7 @@
         <v>55</v>
       </c>
       <c r="K258" s="7">
-        <v>808</v>
+        <v>757</v>
       </c>
       <c r="L258" s="5" t="s">
         <v>17</v>
@@ -12844,7 +12844,7 @@
         <v>59</v>
       </c>
       <c r="K259" s="8">
-        <v>563</v>
+        <v>591</v>
       </c>
       <c r="L259" s="5" t="s">
         <v>17</v>
@@ -12882,7 +12882,7 @@
         <v>51</v>
       </c>
       <c r="K260" s="7">
-        <v>713</v>
+        <v>401</v>
       </c>
       <c r="L260" s="5" t="s">
         <v>17</v>
@@ -12920,7 +12920,7 @@
         <v>55</v>
       </c>
       <c r="K261" s="8">
-        <v>566</v>
+        <v>131</v>
       </c>
       <c r="L261" s="5" t="s">
         <v>17</v>
@@ -12958,7 +12958,7 @@
         <v>59</v>
       </c>
       <c r="K262" s="7">
-        <v>404</v>
+        <v>151</v>
       </c>
       <c r="L262" s="5" t="s">
         <v>17</v>
@@ -12996,7 +12996,7 @@
         <v>51</v>
       </c>
       <c r="K263" s="8">
-        <v>374</v>
+        <v>480</v>
       </c>
       <c r="L263" s="5" t="s">
         <v>17</v>
@@ -13034,7 +13034,7 @@
         <v>55</v>
       </c>
       <c r="K264" s="7">
-        <v>276</v>
+        <v>502</v>
       </c>
       <c r="L264" s="5" t="s">
         <v>17</v>
@@ -13072,7 +13072,7 @@
         <v>59</v>
       </c>
       <c r="K265" s="8">
-        <v>282</v>
+        <v>936</v>
       </c>
       <c r="L265" s="5" t="s">
         <v>17</v>
@@ -13110,7 +13110,7 @@
         <v>51</v>
       </c>
       <c r="K266" s="7">
-        <v>539</v>
+        <v>141</v>
       </c>
       <c r="L266" s="5" t="s">
         <v>17</v>
@@ -13148,7 +13148,7 @@
         <v>55</v>
       </c>
       <c r="K267" s="8">
-        <v>189</v>
+        <v>515</v>
       </c>
       <c r="L267" s="5" t="s">
         <v>17</v>
@@ -13186,7 +13186,7 @@
         <v>59</v>
       </c>
       <c r="K268" s="7">
-        <v>566</v>
+        <v>333</v>
       </c>
       <c r="L268" s="10" t="s">
         <v>244</v>
@@ -13224,7 +13224,7 @@
         <v>51</v>
       </c>
       <c r="K269" s="8">
-        <v>750</v>
+        <v>228</v>
       </c>
       <c r="L269" s="5" t="s">
         <v>17</v>
@@ -13262,7 +13262,7 @@
         <v>55</v>
       </c>
       <c r="K270" s="7">
-        <v>609</v>
+        <v>251</v>
       </c>
       <c r="L270" s="5" t="s">
         <v>17</v>
@@ -13300,7 +13300,7 @@
         <v>59</v>
       </c>
       <c r="K271" s="8">
-        <v>308</v>
+        <v>225</v>
       </c>
       <c r="L271" s="5" t="s">
         <v>17</v>
@@ -13338,7 +13338,7 @@
         <v>51</v>
       </c>
       <c r="K272" s="7">
-        <v>848</v>
+        <v>911</v>
       </c>
       <c r="L272" s="5" t="s">
         <v>17</v>
@@ -13376,7 +13376,7 @@
         <v>55</v>
       </c>
       <c r="K273" s="8">
-        <v>716</v>
+        <v>775</v>
       </c>
       <c r="L273" s="5" t="s">
         <v>17</v>
@@ -13414,7 +13414,7 @@
         <v>59</v>
       </c>
       <c r="K274" s="7">
-        <v>716</v>
+        <v>144</v>
       </c>
       <c r="L274" s="5" t="s">
         <v>17</v>
@@ -13452,7 +13452,7 @@
         <v>51</v>
       </c>
       <c r="K275" s="8">
-        <v>727</v>
+        <v>934</v>
       </c>
       <c r="L275" s="5" t="s">
         <v>17</v>
@@ -13490,7 +13490,7 @@
         <v>55</v>
       </c>
       <c r="K276" s="7">
-        <v>622</v>
+        <v>949</v>
       </c>
       <c r="L276" s="5" t="s">
         <v>17</v>
@@ -13528,7 +13528,7 @@
         <v>59</v>
       </c>
       <c r="K277" s="8">
-        <v>693</v>
+        <v>721</v>
       </c>
       <c r="L277" s="5" t="s">
         <v>17</v>
@@ -13566,7 +13566,7 @@
         <v>51</v>
       </c>
       <c r="K278" s="7">
-        <v>449</v>
+        <v>322</v>
       </c>
       <c r="L278" s="5" t="s">
         <v>17</v>
@@ -13604,7 +13604,7 @@
         <v>55</v>
       </c>
       <c r="K279" s="8">
-        <v>128</v>
+        <v>212</v>
       </c>
       <c r="L279" s="5" t="s">
         <v>17</v>
@@ -13642,7 +13642,7 @@
         <v>59</v>
       </c>
       <c r="K280" s="7">
-        <v>771</v>
+        <v>846</v>
       </c>
       <c r="L280" s="5" t="s">
         <v>17</v>
@@ -13680,7 +13680,7 @@
         <v>51</v>
       </c>
       <c r="K281" s="8">
-        <v>148</v>
+        <v>410</v>
       </c>
       <c r="L281" s="5" t="s">
         <v>17</v>
@@ -13718,7 +13718,7 @@
         <v>55</v>
       </c>
       <c r="K282" s="7">
-        <v>547</v>
+        <v>202</v>
       </c>
       <c r="L282" s="5" t="s">
         <v>17</v>
@@ -13756,7 +13756,7 @@
         <v>59</v>
       </c>
       <c r="K283" s="8">
-        <v>508</v>
+        <v>859</v>
       </c>
       <c r="L283" s="5" t="s">
         <v>17</v>
@@ -13794,7 +13794,7 @@
         <v>51</v>
       </c>
       <c r="K284" s="7">
-        <v>708</v>
+        <v>532</v>
       </c>
       <c r="L284" s="5" t="s">
         <v>17</v>
@@ -13832,7 +13832,7 @@
         <v>55</v>
       </c>
       <c r="K285" s="8">
-        <v>855</v>
+        <v>823</v>
       </c>
       <c r="L285" s="5" t="s">
         <v>17</v>
@@ -13870,7 +13870,7 @@
         <v>59</v>
       </c>
       <c r="K286" s="7">
-        <v>350</v>
+        <v>754</v>
       </c>
       <c r="L286" s="5" t="s">
         <v>17</v>
@@ -13908,7 +13908,7 @@
         <v>51</v>
       </c>
       <c r="K287" s="8">
-        <v>449</v>
+        <v>626</v>
       </c>
       <c r="L287" s="5" t="s">
         <v>17</v>
@@ -13946,7 +13946,7 @@
         <v>55</v>
       </c>
       <c r="K288" s="7">
-        <v>425</v>
+        <v>559</v>
       </c>
       <c r="L288" s="9" t="s">
         <v>142</v>
@@ -13984,7 +13984,7 @@
         <v>59</v>
       </c>
       <c r="K289" s="8">
-        <v>656</v>
+        <v>792</v>
       </c>
       <c r="L289" s="5" t="s">
         <v>17</v>
@@ -14022,7 +14022,7 @@
         <v>51</v>
       </c>
       <c r="K290" s="7">
-        <v>774</v>
+        <v>185</v>
       </c>
       <c r="L290" s="5" t="s">
         <v>17</v>
@@ -14060,7 +14060,7 @@
         <v>55</v>
       </c>
       <c r="K291" s="8">
-        <v>857</v>
+        <v>457</v>
       </c>
       <c r="L291" s="5" t="s">
         <v>17</v>
@@ -14098,7 +14098,7 @@
         <v>59</v>
       </c>
       <c r="K292" s="7">
-        <v>197</v>
+        <v>628</v>
       </c>
       <c r="L292" s="5" t="s">
         <v>17</v>
@@ -14136,7 +14136,7 @@
         <v>51</v>
       </c>
       <c r="K293" s="8">
-        <v>253</v>
+        <v>162</v>
       </c>
       <c r="L293" s="5" t="s">
         <v>17</v>
@@ -14174,7 +14174,7 @@
         <v>55</v>
       </c>
       <c r="K294" s="7">
-        <v>465</v>
+        <v>479</v>
       </c>
       <c r="L294" s="5" t="s">
         <v>17</v>
@@ -14212,7 +14212,7 @@
         <v>59</v>
       </c>
       <c r="K295" s="8">
-        <v>443</v>
+        <v>582</v>
       </c>
       <c r="L295" s="5" t="s">
         <v>17</v>
@@ -14250,7 +14250,7 @@
         <v>51</v>
       </c>
       <c r="K296" s="7">
-        <v>300</v>
+        <v>325</v>
       </c>
       <c r="L296" s="5" t="s">
         <v>17</v>
@@ -14288,7 +14288,7 @@
         <v>55</v>
       </c>
       <c r="K297" s="8">
-        <v>581</v>
+        <v>671</v>
       </c>
       <c r="L297" s="5" t="s">
         <v>17</v>
@@ -14326,7 +14326,7 @@
         <v>59</v>
       </c>
       <c r="K298" s="7">
-        <v>144</v>
+        <v>703</v>
       </c>
       <c r="L298" s="5" t="s">
         <v>17</v>
@@ -14364,7 +14364,7 @@
         <v>51</v>
       </c>
       <c r="K299" s="8">
-        <v>646</v>
+        <v>454</v>
       </c>
       <c r="L299" s="5" t="s">
         <v>17</v>
@@ -14402,7 +14402,7 @@
         <v>55</v>
       </c>
       <c r="K300" s="7">
-        <v>187</v>
+        <v>520</v>
       </c>
       <c r="L300" s="5" t="s">
         <v>17</v>
@@ -14440,7 +14440,7 @@
         <v>59</v>
       </c>
       <c r="K301" s="8">
-        <v>885</v>
+        <v>216</v>
       </c>
       <c r="L301" s="5" t="s">
         <v>17</v>
@@ -14478,7 +14478,7 @@
         <v>51</v>
       </c>
       <c r="K302" s="7">
-        <v>565</v>
+        <v>944</v>
       </c>
       <c r="L302" s="5" t="s">
         <v>17</v>
@@ -14516,7 +14516,7 @@
         <v>55</v>
       </c>
       <c r="K303" s="8">
-        <v>408</v>
+        <v>496</v>
       </c>
       <c r="L303" s="5" t="s">
         <v>17</v>
@@ -14554,7 +14554,7 @@
         <v>59</v>
       </c>
       <c r="K304" s="7">
-        <v>414</v>
+        <v>909</v>
       </c>
       <c r="L304" s="5" t="s">
         <v>17</v>
@@ -14592,7 +14592,7 @@
         <v>51</v>
       </c>
       <c r="K305" s="8">
-        <v>288</v>
+        <v>322</v>
       </c>
       <c r="L305" s="5" t="s">
         <v>17</v>
@@ -14630,7 +14630,7 @@
         <v>55</v>
       </c>
       <c r="K306" s="7">
-        <v>276</v>
+        <v>932</v>
       </c>
       <c r="L306" s="5" t="s">
         <v>17</v>

</xml_diff>